<commit_message>
Superatoms big set: rebuild and publish
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/published_runs/sonnet55_api_superatoms/cxmolscribe/Completed_HighConfidence_CMAGE.xlsx
+++ b/benchmarks/published_runs/sonnet55_api_superatoms/cxmolscribe/Completed_HighConfidence_CMAGE.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1687"/>
+  <dimension ref="A1:K1751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49374,6 +49374,1862 @@
       </c>
       <c r="K1687" t="inlineStr"/>
     </row>
+    <row r="1688">
+      <c r="A1688" s="1" t="n">
+        <v>1686</v>
+      </c>
+      <c r="B1688" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0006.png</t>
+        </is>
+      </c>
+      <c r="C1688" t="inlineStr"/>
+      <c r="D1688" t="inlineStr"/>
+      <c r="E1688" t="inlineStr"/>
+      <c r="F1688" t="inlineStr">
+        <is>
+          <t>O=C(NC(Cc1ccc(OCc2ccccc2)nc1)C(=O)N1CCC(N2CCCCC2)CC1)N1CCC(N2Cc3ccccc3NC2=O)CC1</t>
+        </is>
+      </c>
+      <c r="G1688" t="inlineStr"/>
+      <c r="H1688" t="inlineStr"/>
+      <c r="I1688" t="n">
+        <v>0.9142170765838024</v>
+      </c>
+      <c r="J1688" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1688" t="inlineStr"/>
+    </row>
+    <row r="1689">
+      <c r="A1689" s="1" t="n">
+        <v>1687</v>
+      </c>
+      <c r="B1689" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0008.png</t>
+        </is>
+      </c>
+      <c r="C1689" t="inlineStr"/>
+      <c r="D1689" t="inlineStr"/>
+      <c r="E1689" t="inlineStr"/>
+      <c r="F1689" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1CC1(NC(=O)[C@@H]1C[C@@H](Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN1C(=O)[C@@H](OC(=O)NC(C)(C)C)C(C)(C)C)C(=O)NS(=O)(=O)C1(CC2CC2)CC1</t>
+        </is>
+      </c>
+      <c r="G1689" t="inlineStr"/>
+      <c r="H1689" t="inlineStr"/>
+      <c r="I1689" t="n">
+        <v>0.9008674185420836</v>
+      </c>
+      <c r="J1689" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1689" t="inlineStr"/>
+    </row>
+    <row r="1690">
+      <c r="A1690" s="1" t="n">
+        <v>1688</v>
+      </c>
+      <c r="B1690" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0009.png</t>
+        </is>
+      </c>
+      <c r="C1690" t="inlineStr"/>
+      <c r="D1690" t="inlineStr"/>
+      <c r="E1690" t="inlineStr"/>
+      <c r="F1690" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@@H](Oc2nccc3ccccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccc(C(C)(C)C)cc1)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1690" t="inlineStr"/>
+      <c r="H1690" t="inlineStr"/>
+      <c r="I1690" t="n">
+        <v>0.9131192918353959</v>
+      </c>
+      <c r="J1690" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1690" t="inlineStr"/>
+    </row>
+    <row r="1691">
+      <c r="A1691" s="1" t="n">
+        <v>1689</v>
+      </c>
+      <c r="B1691" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0011.png</t>
+        </is>
+      </c>
+      <c r="C1691" t="inlineStr"/>
+      <c r="D1691" t="inlineStr"/>
+      <c r="E1691" t="inlineStr"/>
+      <c r="F1691" t="inlineStr">
+        <is>
+          <t>NC(CCC(=O)NCCCC(=O)N[C@@H](CNC(=O)c1ccc2c(cnn2CCCNc2ncc[nH]2)c1)C(=O)O)C(=O)NCCCCCC(=O)N[C@@H](CNC(=O)c1ccc2c(cnn2CCCNc2ncc[nH]2)c1)C(=O)O</t>
+        </is>
+      </c>
+      <c r="G1691" t="inlineStr"/>
+      <c r="H1691" t="inlineStr"/>
+      <c r="I1691" t="n">
+        <v>0.9059905721446931</v>
+      </c>
+      <c r="J1691" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1691" t="inlineStr"/>
+    </row>
+    <row r="1692">
+      <c r="A1692" s="1" t="n">
+        <v>1690</v>
+      </c>
+      <c r="B1692" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0013.png</t>
+        </is>
+      </c>
+      <c r="C1692" t="inlineStr"/>
+      <c r="D1692" t="inlineStr"/>
+      <c r="E1692" t="inlineStr"/>
+      <c r="F1692" t="inlineStr">
+        <is>
+          <t>Cc1cc(OCCCC(=O)NCCNC(=O)C(CCC(=O)OC(C)(C)C)NC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)OCc2ccccc2)cc(C)c1S(=O)(=O)N[C@@H](CNC(=O)c1ccc2c(cnn2CCCNc2ncc[nH]2)c1)C(=O)O</t>
+        </is>
+      </c>
+      <c r="G1692" t="inlineStr"/>
+      <c r="H1692" t="inlineStr"/>
+      <c r="I1692" t="n">
+        <v>0.8972030700707886</v>
+      </c>
+      <c r="J1692" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1692" t="inlineStr"/>
+    </row>
+    <row r="1693">
+      <c r="A1693" s="1" t="n">
+        <v>1691</v>
+      </c>
+      <c r="B1693" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0014.png</t>
+        </is>
+      </c>
+      <c r="C1693" t="inlineStr"/>
+      <c r="D1693" t="inlineStr"/>
+      <c r="E1693" t="inlineStr"/>
+      <c r="F1693" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@H](Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccc(OC)cc1)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1693" t="inlineStr"/>
+      <c r="H1693" t="inlineStr"/>
+      <c r="I1693" t="n">
+        <v>0.9073033447622657</v>
+      </c>
+      <c r="J1693" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1693" t="inlineStr"/>
+    </row>
+    <row r="1694">
+      <c r="A1694" s="1" t="n">
+        <v>1692</v>
+      </c>
+      <c r="B1694" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0015.png</t>
+        </is>
+      </c>
+      <c r="C1694" t="inlineStr"/>
+      <c r="D1694" t="inlineStr"/>
+      <c r="E1694" t="inlineStr"/>
+      <c r="F1694" t="inlineStr">
+        <is>
+          <t>c1cc(-c2ccc3ccc4cccnc4c3n2)cc(-c2ccccc2-c2ccccc2-c2cccc(-c3ccc4ccc5cccnc5c4n3)c2)c1</t>
+        </is>
+      </c>
+      <c r="G1694" t="inlineStr"/>
+      <c r="H1694" t="inlineStr"/>
+      <c r="I1694" t="n">
+        <v>0.9210780030190178</v>
+      </c>
+      <c r="J1694" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1694" t="inlineStr"/>
+    </row>
+    <row r="1695">
+      <c r="A1695" s="1" t="n">
+        <v>1693</v>
+      </c>
+      <c r="B1695" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0016.png</t>
+        </is>
+      </c>
+      <c r="C1695" t="inlineStr"/>
+      <c r="D1695" t="inlineStr"/>
+      <c r="E1695" t="inlineStr"/>
+      <c r="F1695" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@H](Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccc(N(C)C)cc1)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1695" t="inlineStr"/>
+      <c r="H1695" t="inlineStr"/>
+      <c r="I1695" t="n">
+        <v>0.8969342911597011</v>
+      </c>
+      <c r="J1695" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1695" t="inlineStr"/>
+    </row>
+    <row r="1696">
+      <c r="A1696" s="1" t="n">
+        <v>1694</v>
+      </c>
+      <c r="B1696" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0019.png</t>
+        </is>
+      </c>
+      <c r="C1696" t="inlineStr"/>
+      <c r="D1696" t="inlineStr"/>
+      <c r="E1696" t="inlineStr"/>
+      <c r="F1696" t="inlineStr">
+        <is>
+          <t>CC1=C(/C=C/C=C/C=C/C=C/C=C/C=C/C=C/C=C(C)/C=C/C2=C(C)C(=O)C(OP(=O)(O)O)CC2(C)C)C(C)(C)CC(OP(=O)(O)O)C1=O</t>
+        </is>
+      </c>
+      <c r="G1696" t="inlineStr"/>
+      <c r="H1696" t="inlineStr"/>
+      <c r="I1696" t="n">
+        <v>0.8858947752673534</v>
+      </c>
+      <c r="J1696" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1696" t="inlineStr"/>
+    </row>
+    <row r="1697">
+      <c r="A1697" s="1" t="n">
+        <v>1695</v>
+      </c>
+      <c r="B1697" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0020.png</t>
+        </is>
+      </c>
+      <c r="C1697" t="inlineStr"/>
+      <c r="D1697" t="inlineStr"/>
+      <c r="E1697" t="inlineStr"/>
+      <c r="F1697" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@@]1(NC(=O)[C@@H]1CC(Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN1C(=O)[C@@H](O)C(C)(C)C)C(=O)NS(=O)(=O)C1(CC2CC2)CC1</t>
+        </is>
+      </c>
+      <c r="G1697" t="inlineStr"/>
+      <c r="H1697" t="inlineStr"/>
+      <c r="I1697" t="n">
+        <v>0.8890468321032035</v>
+      </c>
+      <c r="J1697" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1697" t="inlineStr"/>
+    </row>
+    <row r="1698">
+      <c r="A1698" s="1" t="n">
+        <v>1696</v>
+      </c>
+      <c r="B1698" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0021.png</t>
+        </is>
+      </c>
+      <c r="C1698" t="inlineStr"/>
+      <c r="D1698" t="inlineStr"/>
+      <c r="E1698" t="inlineStr"/>
+      <c r="F1698" t="inlineStr">
+        <is>
+          <t>[H][C@]1(Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN(C(=O)[C@]([H])(O)c2ccccc2)[C@]([H])(C(=O)N[C@]2(C(=O)NS(=O)(=O)C3CC3)C[C@@]2([H])C=C)C1</t>
+        </is>
+      </c>
+      <c r="G1698" t="inlineStr"/>
+      <c r="H1698" t="inlineStr"/>
+      <c r="I1698" t="n">
+        <v>0.8899591704481401</v>
+      </c>
+      <c r="J1698" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1698" t="inlineStr"/>
+    </row>
+    <row r="1699">
+      <c r="A1699" s="1" t="n">
+        <v>1697</v>
+      </c>
+      <c r="B1699" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0022.png</t>
+        </is>
+      </c>
+      <c r="C1699" t="inlineStr"/>
+      <c r="D1699" t="inlineStr"/>
+      <c r="E1699" t="inlineStr"/>
+      <c r="F1699" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(cnn2CCCNc2ncccn2)c1)NS(=O)(=O)c1c(C)cc(OCCCC(=O)NCCNC(=O)OCc2ccccc2)cc1C</t>
+        </is>
+      </c>
+      <c r="G1699" t="inlineStr"/>
+      <c r="H1699" t="inlineStr"/>
+      <c r="I1699" t="n">
+        <v>0.8942836240659651</v>
+      </c>
+      <c r="J1699" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1699" t="inlineStr"/>
+    </row>
+    <row r="1700">
+      <c r="A1700" s="1" t="n">
+        <v>1698</v>
+      </c>
+      <c r="B1700" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0023.png</t>
+        </is>
+      </c>
+      <c r="C1700" t="inlineStr"/>
+      <c r="D1700" t="inlineStr"/>
+      <c r="E1700" t="inlineStr"/>
+      <c r="F1700" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(CCCNC3=NCCCC3)nn(C)c2c1)NS(=O)(=O)c1c(C)cc(OCCCC(=O)NCCNC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)OCc2ccccc2)cc1C</t>
+        </is>
+      </c>
+      <c r="G1700" t="inlineStr"/>
+      <c r="H1700" t="inlineStr"/>
+      <c r="I1700" t="n">
+        <v>0.8938599646997502</v>
+      </c>
+      <c r="J1700" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1700" t="inlineStr"/>
+    </row>
+    <row r="1701">
+      <c r="A1701" s="1" t="n">
+        <v>1699</v>
+      </c>
+      <c r="B1701" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0024.png</t>
+        </is>
+      </c>
+      <c r="C1701" t="inlineStr"/>
+      <c r="D1701" t="inlineStr"/>
+      <c r="E1701" t="inlineStr"/>
+      <c r="F1701" t="inlineStr">
+        <is>
+          <t>C=CC1CC1(NC(=O)[C@@H]1CC(Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccc(OC)cc1C)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1701" t="inlineStr"/>
+      <c r="H1701" t="inlineStr"/>
+      <c r="I1701" t="n">
+        <v>0.9159639749347586</v>
+      </c>
+      <c r="J1701" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1701" t="inlineStr"/>
+    </row>
+    <row r="1702">
+      <c r="A1702" s="1" t="n">
+        <v>1700</v>
+      </c>
+      <c r="B1702" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0025.png</t>
+        </is>
+      </c>
+      <c r="C1702" t="inlineStr"/>
+      <c r="D1702" t="inlineStr"/>
+      <c r="E1702" t="inlineStr"/>
+      <c r="F1702" t="inlineStr">
+        <is>
+          <t>CC1(C)O[C@@H]2[C@H](O1)[C@@H](/C=C/CNC(=O)c1cc(C(=O)c3ccncc3)cc3c1OC(c1ccccc1)(c1ccccc1)O3)O[C@H]2n1cnc2c(N)ncnc21</t>
+        </is>
+      </c>
+      <c r="G1702" t="inlineStr"/>
+      <c r="H1702" t="inlineStr"/>
+      <c r="I1702" t="n">
+        <v>0.896823333093274</v>
+      </c>
+      <c r="J1702" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1702" t="inlineStr"/>
+    </row>
+    <row r="1703">
+      <c r="A1703" s="1" t="n">
+        <v>1701</v>
+      </c>
+      <c r="B1703" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0026.png</t>
+        </is>
+      </c>
+      <c r="C1703" t="inlineStr"/>
+      <c r="D1703" t="inlineStr"/>
+      <c r="E1703" t="inlineStr"/>
+      <c r="F1703" t="inlineStr">
+        <is>
+          <t>CC1(C)O[C@@H]2[C@H](O1)[C@@H](/C=C/CNC(=O)c1cc(-c3nccs3)cc3c1OC(c1ccccc1)(c1ccccc1)O3)O[C@H]2n1cnc2c(N)ncnc21</t>
+        </is>
+      </c>
+      <c r="G1703" t="inlineStr"/>
+      <c r="H1703" t="inlineStr"/>
+      <c r="I1703" t="n">
+        <v>0.8915959474653408</v>
+      </c>
+      <c r="J1703" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1703" t="inlineStr"/>
+    </row>
+    <row r="1704">
+      <c r="A1704" s="1" t="n">
+        <v>1702</v>
+      </c>
+      <c r="B1704" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0030.png</t>
+        </is>
+      </c>
+      <c r="C1704" t="inlineStr"/>
+      <c r="D1704" t="inlineStr"/>
+      <c r="E1704" t="inlineStr"/>
+      <c r="F1704" t="inlineStr">
+        <is>
+          <t>CC1(C)O[C@@H]2[C@H](O1)[C@H](n1cnc3c(N)ncnc31)O[C@@H]2/C=C/CNC(=O)c1cc(-c2nc3ccccc3s2)cc2c1OC(c1ccccc1)(c1ccccc1)O2</t>
+        </is>
+      </c>
+      <c r="G1704" t="inlineStr"/>
+      <c r="H1704" t="inlineStr"/>
+      <c r="I1704" t="n">
+        <v>0.8870881154821409</v>
+      </c>
+      <c r="J1704" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1704" t="inlineStr"/>
+    </row>
+    <row r="1705">
+      <c r="A1705" s="1" t="n">
+        <v>1703</v>
+      </c>
+      <c r="B1705" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0031.png</t>
+        </is>
+      </c>
+      <c r="C1705" t="inlineStr"/>
+      <c r="D1705" t="inlineStr"/>
+      <c r="E1705" t="inlineStr"/>
+      <c r="F1705" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@@H](Oc2nccc3ccccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccc(F)cc1)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1705" t="inlineStr"/>
+      <c r="H1705" t="inlineStr"/>
+      <c r="I1705" t="n">
+        <v>0.9097663454707612</v>
+      </c>
+      <c r="J1705" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1705" t="inlineStr"/>
+    </row>
+    <row r="1706">
+      <c r="A1706" s="1" t="n">
+        <v>1704</v>
+      </c>
+      <c r="B1706" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0032.png</t>
+        </is>
+      </c>
+      <c r="C1706" t="inlineStr"/>
+      <c r="D1706" t="inlineStr"/>
+      <c r="E1706" t="inlineStr"/>
+      <c r="F1706" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(cnn2CCNC2=NCCCC2)c1)NS(=O)(=O)c1ccc(-c2ccc(S(=O)(=O)NCCNC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)OCc3ccccc3)cc2)cc1</t>
+        </is>
+      </c>
+      <c r="G1706" t="inlineStr"/>
+      <c r="H1706" t="inlineStr"/>
+      <c r="I1706" t="n">
+        <v>0.8847456761217281</v>
+      </c>
+      <c r="J1706" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1706" t="inlineStr"/>
+    </row>
+    <row r="1707">
+      <c r="A1707" s="1" t="n">
+        <v>1705</v>
+      </c>
+      <c r="B1707" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0033.png</t>
+        </is>
+      </c>
+      <c r="C1707" t="inlineStr"/>
+      <c r="D1707" t="inlineStr"/>
+      <c r="E1707" t="inlineStr"/>
+      <c r="F1707" t="inlineStr">
+        <is>
+          <t>Cc1cc(OCCCC(=O)NCCNC(=O)C(CCC(=O)OC(C)(C)C)NC(=O)[C@@H](N)CCC(=O)OC(C)(C)C)cc(C)c1S(=O)(=O)N[C@@H](CNC(=O)c1ccc2c(cnn2CCCNc2ncc[nH]2)c1)C(=O)O</t>
+        </is>
+      </c>
+      <c r="G1707" t="inlineStr"/>
+      <c r="H1707" t="inlineStr"/>
+      <c r="I1707" t="n">
+        <v>0.880686318362027</v>
+      </c>
+      <c r="J1707" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1707" t="inlineStr"/>
+    </row>
+    <row r="1708">
+      <c r="A1708" s="1" t="n">
+        <v>1706</v>
+      </c>
+      <c r="B1708" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0035.png</t>
+        </is>
+      </c>
+      <c r="C1708" t="inlineStr"/>
+      <c r="D1708" t="inlineStr"/>
+      <c r="E1708" t="inlineStr"/>
+      <c r="F1708" t="inlineStr">
+        <is>
+          <t>Cc1ccc(Cc2cc3c(c(C(=O)NC/C=C/[C@H]4O[C@@H](n5cnc6c(N)ncnc65)[C@@H]5OC(C)(C)OC54)c2)OC(c2ccccc2)(c2ccccc2)O3)cc1</t>
+        </is>
+      </c>
+      <c r="G1708" t="inlineStr"/>
+      <c r="H1708" t="inlineStr"/>
+      <c r="I1708" t="n">
+        <v>0.902444519862141</v>
+      </c>
+      <c r="J1708" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1708" t="inlineStr"/>
+    </row>
+    <row r="1709">
+      <c r="A1709" s="1" t="n">
+        <v>1707</v>
+      </c>
+      <c r="B1709" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0036.png</t>
+        </is>
+      </c>
+      <c r="C1709" t="inlineStr"/>
+      <c r="D1709" t="inlineStr"/>
+      <c r="E1709" t="inlineStr"/>
+      <c r="F1709" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(cnn2CCCNC2=NCCCN2)c1)NS(=O)(=O)c1ccc(-c2ccc(S(=O)(=O)NCCNC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)OCc3ccccc3)cc2)cc1</t>
+        </is>
+      </c>
+      <c r="G1709" t="inlineStr"/>
+      <c r="H1709" t="inlineStr"/>
+      <c r="I1709" t="n">
+        <v>0.8955557204829121</v>
+      </c>
+      <c r="J1709" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1709" t="inlineStr"/>
+    </row>
+    <row r="1710">
+      <c r="A1710" s="1" t="n">
+        <v>1708</v>
+      </c>
+      <c r="B1710" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0037.png</t>
+        </is>
+      </c>
+      <c r="C1710" t="inlineStr"/>
+      <c r="D1710" t="inlineStr"/>
+      <c r="E1710" t="inlineStr"/>
+      <c r="F1710" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(cnn2CCCNC2=NCCCN2)c1)NS(=O)(=O)c1c(C)cc(OCCCC(=O)NCCNC(=O)C(N)CCC(=O)OC(C)(C)C)cc1C</t>
+        </is>
+      </c>
+      <c r="G1710" t="inlineStr"/>
+      <c r="H1710" t="inlineStr"/>
+      <c r="I1710" t="n">
+        <v>0.8892282666557172</v>
+      </c>
+      <c r="J1710" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1710" t="inlineStr"/>
+    </row>
+    <row r="1711">
+      <c r="A1711" s="1" t="n">
+        <v>1709</v>
+      </c>
+      <c r="B1711" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0038.png</t>
+        </is>
+      </c>
+      <c r="C1711" t="inlineStr"/>
+      <c r="D1711" t="inlineStr"/>
+      <c r="E1711" t="inlineStr"/>
+      <c r="F1711" t="inlineStr">
+        <is>
+          <t>CC1(C)O[C@@H]2[C@H](O1)[C@@H](/C=C/CNC(=O)c1cc(-c3ccncc3)cc3c1OC(c1ccccc1)(c1ccccc1)O3)O[C@H]2n1cnc2c(N)ncnc21</t>
+        </is>
+      </c>
+      <c r="G1711" t="inlineStr"/>
+      <c r="H1711" t="inlineStr"/>
+      <c r="I1711" t="n">
+        <v>0.8944543207967235</v>
+      </c>
+      <c r="J1711" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1711" t="inlineStr"/>
+    </row>
+    <row r="1712">
+      <c r="A1712" s="1" t="n">
+        <v>1710</v>
+      </c>
+      <c r="B1712" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0041.png</t>
+        </is>
+      </c>
+      <c r="C1712" t="inlineStr"/>
+      <c r="D1712" t="inlineStr"/>
+      <c r="E1712" t="inlineStr"/>
+      <c r="F1712" t="inlineStr">
+        <is>
+          <t>CC(C)(C)OC(=O)n1ncc2cc(CC(CC(=O)N3CCC(N4Cc5ccccc5NC4=O)CC3)C(=O)N3CCC(N4CCCCC4)CC3)ccc21</t>
+        </is>
+      </c>
+      <c r="G1712" t="inlineStr"/>
+      <c r="H1712" t="inlineStr"/>
+      <c r="I1712" t="n">
+        <v>0.9199019996272951</v>
+      </c>
+      <c r="J1712" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1712" t="inlineStr"/>
+    </row>
+    <row r="1713">
+      <c r="A1713" s="1" t="n">
+        <v>1711</v>
+      </c>
+      <c r="B1713" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0042.png</t>
+        </is>
+      </c>
+      <c r="C1713" t="inlineStr"/>
+      <c r="D1713" t="inlineStr"/>
+      <c r="E1713" t="inlineStr"/>
+      <c r="F1713" t="inlineStr">
+        <is>
+          <t>Cc1cc(C)cc(-c2[nH]c3sc(C(C)(C)C(=O)N4C5CCC4CC5)cc3c2[C@H](C)CN/C(=N/C(=O)OC(C)C)N2CCN(c3ccncc3)CC2)c1</t>
+        </is>
+      </c>
+      <c r="G1713" t="inlineStr"/>
+      <c r="H1713" t="inlineStr"/>
+      <c r="I1713" t="n">
+        <v>0.8949040905954962</v>
+      </c>
+      <c r="J1713" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1713" t="inlineStr"/>
+    </row>
+    <row r="1714">
+      <c r="A1714" s="1" t="n">
+        <v>1712</v>
+      </c>
+      <c r="B1714" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0046.png</t>
+        </is>
+      </c>
+      <c r="C1714" t="inlineStr"/>
+      <c r="D1714" t="inlineStr"/>
+      <c r="E1714" t="inlineStr"/>
+      <c r="F1714" t="inlineStr">
+        <is>
+          <t>CC[C@H]1C[C@]1(NC(=O)[C@@H]1C[C@@H](Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN1C(=O)C(O)Cc1c[nH]cn1)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1714" t="inlineStr"/>
+      <c r="H1714" t="inlineStr"/>
+      <c r="I1714" t="n">
+        <v>0.9076067119803672</v>
+      </c>
+      <c r="J1714" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1714" t="inlineStr"/>
+    </row>
+    <row r="1715">
+      <c r="A1715" s="1" t="n">
+        <v>1713</v>
+      </c>
+      <c r="B1715" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0047.png</t>
+        </is>
+      </c>
+      <c r="C1715" t="inlineStr"/>
+      <c r="D1715" t="inlineStr"/>
+      <c r="E1715" t="inlineStr"/>
+      <c r="F1715" t="inlineStr">
+        <is>
+          <t>Cc1cc(C)cc(-c2[nH]c3sc(C(C)(C)C(=O)N4C5CCC4CC5)cc3c2CCN/C(=N/C(=O)OC(C)C)N2CCC(c3ccncc3)C2)c1</t>
+        </is>
+      </c>
+      <c r="G1715" t="inlineStr"/>
+      <c r="H1715" t="inlineStr"/>
+      <c r="I1715" t="n">
+        <v>0.889653278681565</v>
+      </c>
+      <c r="J1715" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1715" t="inlineStr"/>
+    </row>
+    <row r="1716">
+      <c r="A1716" s="1" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B1716" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0048.png</t>
+        </is>
+      </c>
+      <c r="C1716" t="inlineStr"/>
+      <c r="D1716" t="inlineStr"/>
+      <c r="E1716" t="inlineStr"/>
+      <c r="F1716" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(cnn2CCCNc2ncccn2)c1)NS(=O)(=O)c1ccc(-c2ccc(S(=O)(=O)NCCNC(=O)OCc3ccccc3)cc2)cc1</t>
+        </is>
+      </c>
+      <c r="G1716" t="inlineStr"/>
+      <c r="H1716" t="inlineStr"/>
+      <c r="I1716" t="n">
+        <v>0.893672977762292</v>
+      </c>
+      <c r="J1716" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1716" t="inlineStr"/>
+    </row>
+    <row r="1717">
+      <c r="A1717" s="1" t="n">
+        <v>1715</v>
+      </c>
+      <c r="B1717" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0049.png</t>
+        </is>
+      </c>
+      <c r="C1717" t="inlineStr"/>
+      <c r="D1717" t="inlineStr"/>
+      <c r="E1717" t="inlineStr"/>
+      <c r="F1717" t="inlineStr">
+        <is>
+          <t>Cc1cc(OCCCC(=O)NCCNC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)OCc2ccccc2)cc(C)c1S(=O)(=O)N[C@@H](CNC(=O)c1ccc2c(cnn2CCNC2=NCCCC2)c1)C(=O)O</t>
+        </is>
+      </c>
+      <c r="G1717" t="inlineStr"/>
+      <c r="H1717" t="inlineStr"/>
+      <c r="I1717" t="n">
+        <v>0.884760816211659</v>
+      </c>
+      <c r="J1717" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1717" t="inlineStr"/>
+    </row>
+    <row r="1718">
+      <c r="A1718" s="1" t="n">
+        <v>1716</v>
+      </c>
+      <c r="B1718" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0050.png</t>
+        </is>
+      </c>
+      <c r="C1718" t="inlineStr"/>
+      <c r="D1718" t="inlineStr"/>
+      <c r="E1718" t="inlineStr"/>
+      <c r="F1718" t="inlineStr">
+        <is>
+          <t>[H][C@]1(Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN(C(=O)C(O)c2ccccc2)[C@]([H])(C(=O)N[C@]2(C(=O)NS(=O)(=O)C3CC3)C[C@@]2([H])C=C)C1</t>
+        </is>
+      </c>
+      <c r="G1718" t="inlineStr"/>
+      <c r="H1718" t="inlineStr"/>
+      <c r="I1718" t="n">
+        <v>0.8953091419398913</v>
+      </c>
+      <c r="J1718" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1718" t="inlineStr"/>
+    </row>
+    <row r="1719">
+      <c r="A1719" s="1" t="n">
+        <v>1717</v>
+      </c>
+      <c r="B1719" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0052.png</t>
+        </is>
+      </c>
+      <c r="C1719" t="inlineStr"/>
+      <c r="D1719" t="inlineStr"/>
+      <c r="E1719" t="inlineStr"/>
+      <c r="F1719" t="inlineStr">
+        <is>
+          <t>C=CC1CC1(NC(=O)[C@@H]1CC(Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccc(OC)cc1)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1719" t="inlineStr"/>
+      <c r="H1719" t="inlineStr"/>
+      <c r="I1719" t="n">
+        <v>0.9160497383125208</v>
+      </c>
+      <c r="J1719" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1719" t="inlineStr"/>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="1" t="n">
+        <v>1718</v>
+      </c>
+      <c r="B1720" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0053.png</t>
+        </is>
+      </c>
+      <c r="C1720" t="inlineStr"/>
+      <c r="D1720" t="inlineStr"/>
+      <c r="E1720" t="inlineStr"/>
+      <c r="F1720" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(cnn2CCCNC2=NCCCN2)c1)NS(=O)(=O)c1c(C)cc(OCCCC(=O)NCCNC(=O)C(CCC(=O)OC(C)(C)C)NC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)OCc2ccccc2)cc1C</t>
+        </is>
+      </c>
+      <c r="G1720" t="inlineStr"/>
+      <c r="H1720" t="inlineStr"/>
+      <c r="I1720" t="n">
+        <v>0.8792676041129015</v>
+      </c>
+      <c r="J1720" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1720" t="inlineStr"/>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="1" t="n">
+        <v>1719</v>
+      </c>
+      <c r="B1721" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0054.png</t>
+        </is>
+      </c>
+      <c r="C1721" t="inlineStr"/>
+      <c r="D1721" t="inlineStr"/>
+      <c r="E1721" t="inlineStr"/>
+      <c r="F1721" t="inlineStr">
+        <is>
+          <t>O=C(NC(Cc1ccc2[nH]ncc2c1)C(=O)N1CCC(N2Cc3ccccc3NC2=O)CC1)N1CCC(N2Cc3ccccc3NC2=O)CC1</t>
+        </is>
+      </c>
+      <c r="G1721" t="inlineStr"/>
+      <c r="H1721" t="inlineStr"/>
+      <c r="I1721" t="n">
+        <v>0.9207033166920465</v>
+      </c>
+      <c r="J1721" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1721" t="inlineStr"/>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="1" t="n">
+        <v>1720</v>
+      </c>
+      <c r="B1722" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0056.png</t>
+        </is>
+      </c>
+      <c r="C1722" t="inlineStr"/>
+      <c r="D1722" t="inlineStr"/>
+      <c r="E1722" t="inlineStr"/>
+      <c r="F1722" t="inlineStr">
+        <is>
+          <t>Cc1cc(C)cc(-c2[nH]c3sc(C(C)(C)C(=O)N4C5CCC4CC5)cc3c2[C@H](C)CN/C(=N/C(=O)OC(C)C)N2CCC(c3ccncc3)CC2)c1</t>
+        </is>
+      </c>
+      <c r="G1722" t="inlineStr"/>
+      <c r="H1722" t="inlineStr"/>
+      <c r="I1722" t="n">
+        <v>0.8960723402285682</v>
+      </c>
+      <c r="J1722" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1722" t="inlineStr"/>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="1" t="n">
+        <v>1721</v>
+      </c>
+      <c r="B1723" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0057.png</t>
+        </is>
+      </c>
+      <c r="C1723" t="inlineStr"/>
+      <c r="D1723" t="inlineStr"/>
+      <c r="E1723" t="inlineStr"/>
+      <c r="F1723" t="inlineStr">
+        <is>
+          <t>CC(=O)c1ccc2c(c1)C1(c3cc(-c4ccc5ccc6ccccc6c5n4)ccc3-2)c2cc(-c3ccc4ccc5ccccc5c4n3)ccc2-c2ccc(-c3ccc4ccc5ccccc5c4n3)cc21</t>
+        </is>
+      </c>
+      <c r="G1723" t="inlineStr"/>
+      <c r="H1723" t="inlineStr"/>
+      <c r="I1723" t="n">
+        <v>0.894957416468548</v>
+      </c>
+      <c r="J1723" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1723" t="inlineStr"/>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="1" t="n">
+        <v>1722</v>
+      </c>
+      <c r="B1724" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0058.png</t>
+        </is>
+      </c>
+      <c r="C1724" t="inlineStr"/>
+      <c r="D1724" t="inlineStr"/>
+      <c r="E1724" t="inlineStr"/>
+      <c r="F1724" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(CCCNc3ccccn3)nn(C)c2c1)NS(=O)(=O)c1c(C)cc(OCCCC(=O)NCCNC(=O)OCc2ccccc2)cc1C</t>
+        </is>
+      </c>
+      <c r="G1724" t="inlineStr"/>
+      <c r="H1724" t="inlineStr"/>
+      <c r="I1724" t="n">
+        <v>0.9033998893373066</v>
+      </c>
+      <c r="J1724" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1724" t="inlineStr"/>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="1" t="n">
+        <v>1723</v>
+      </c>
+      <c r="B1725" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0060.png</t>
+        </is>
+      </c>
+      <c r="C1725" t="inlineStr"/>
+      <c r="D1725" t="inlineStr"/>
+      <c r="E1725" t="inlineStr"/>
+      <c r="F1725" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@@H](Oc2nccc3ccccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccccc1OC)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1725" t="inlineStr"/>
+      <c r="H1725" t="inlineStr"/>
+      <c r="I1725" t="n">
+        <v>0.9023607108190183</v>
+      </c>
+      <c r="J1725" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1725" t="inlineStr"/>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="1" t="n">
+        <v>1724</v>
+      </c>
+      <c r="B1726" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0062.png</t>
+        </is>
+      </c>
+      <c r="C1726" t="inlineStr"/>
+      <c r="D1726" t="inlineStr"/>
+      <c r="E1726" t="inlineStr"/>
+      <c r="F1726" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@@H](Oc2cc(-c3cccs3)cc(-c3ccccc3)n2)CN1C(=O)[C@@H](OC(=O)NC(C)(C)C)C(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1726" t="inlineStr"/>
+      <c r="H1726" t="inlineStr"/>
+      <c r="I1726" t="n">
+        <v>0.9001725000769537</v>
+      </c>
+      <c r="J1726" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1726" t="inlineStr"/>
+    </row>
+    <row r="1727">
+      <c r="A1727" s="1" t="n">
+        <v>1725</v>
+      </c>
+      <c r="B1727" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0065.png</t>
+        </is>
+      </c>
+      <c r="C1727" t="inlineStr"/>
+      <c r="D1727" t="inlineStr"/>
+      <c r="E1727" t="inlineStr"/>
+      <c r="F1727" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@H](Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccc(OC)cc1C)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1727" t="inlineStr"/>
+      <c r="H1727" t="inlineStr"/>
+      <c r="I1727" t="n">
+        <v>0.9065342442348568</v>
+      </c>
+      <c r="J1727" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1727" t="inlineStr"/>
+    </row>
+    <row r="1728">
+      <c r="A1728" s="1" t="n">
+        <v>1726</v>
+      </c>
+      <c r="B1728" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0067.png</t>
+        </is>
+      </c>
+      <c r="C1728" t="inlineStr"/>
+      <c r="D1728" t="inlineStr"/>
+      <c r="E1728" t="inlineStr"/>
+      <c r="F1728" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@@H](Oc2nccc3ccccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccc(OC)cc1)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1728" t="inlineStr"/>
+      <c r="H1728" t="inlineStr"/>
+      <c r="I1728" t="n">
+        <v>0.9083649568773515</v>
+      </c>
+      <c r="J1728" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1728" t="inlineStr"/>
+    </row>
+    <row r="1729">
+      <c r="A1729" s="1" t="n">
+        <v>1727</v>
+      </c>
+      <c r="B1729" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0068.png</t>
+        </is>
+      </c>
+      <c r="C1729" t="inlineStr"/>
+      <c r="D1729" t="inlineStr"/>
+      <c r="E1729" t="inlineStr"/>
+      <c r="F1729" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@@H](Oc2nc(-c3ccc(OC(F)(F)F)cc3)cc3cc(OC)ccc23)CN1C(=O)[C@@H](OC(=O)NC(C)(C)C)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1729" t="inlineStr"/>
+      <c r="H1729" t="inlineStr"/>
+      <c r="I1729" t="n">
+        <v>0.8955345356250366</v>
+      </c>
+      <c r="J1729" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1729" t="inlineStr"/>
+    </row>
+    <row r="1730">
+      <c r="A1730" s="1" t="n">
+        <v>1728</v>
+      </c>
+      <c r="B1730" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0069.png</t>
+        </is>
+      </c>
+      <c r="C1730" t="inlineStr"/>
+      <c r="D1730" t="inlineStr"/>
+      <c r="E1730" t="inlineStr"/>
+      <c r="F1730" t="inlineStr">
+        <is>
+          <t>Cc1cc(C)cc(-c2[nH]c3sc(C(C)(C)C(=O)N4C5CCC4CC5)cc3c2[C@H](C)CN/C(=N/C(=O)OC(C)C)N2CCC(c3ccccn3)C2)c1</t>
+        </is>
+      </c>
+      <c r="G1730" t="inlineStr"/>
+      <c r="H1730" t="inlineStr"/>
+      <c r="I1730" t="n">
+        <v>0.8951914024924019</v>
+      </c>
+      <c r="J1730" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1730" t="inlineStr"/>
+    </row>
+    <row r="1731">
+      <c r="A1731" s="1" t="n">
+        <v>1729</v>
+      </c>
+      <c r="B1731" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0070.png</t>
+        </is>
+      </c>
+      <c r="C1731" t="inlineStr"/>
+      <c r="D1731" t="inlineStr"/>
+      <c r="E1731" t="inlineStr"/>
+      <c r="F1731" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@@H](Oc2nccc3ccccc23)CN1C(=O)[C@@H](OC(=O)Nc1ccccc1C(C)C)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1731" t="inlineStr"/>
+      <c r="H1731" t="inlineStr"/>
+      <c r="I1731" t="n">
+        <v>0.881482076679066</v>
+      </c>
+      <c r="J1731" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1731" t="inlineStr"/>
+    </row>
+    <row r="1732">
+      <c r="A1732" s="1" t="n">
+        <v>1730</v>
+      </c>
+      <c r="B1732" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0071.png</t>
+        </is>
+      </c>
+      <c r="C1732" t="inlineStr"/>
+      <c r="D1732" t="inlineStr"/>
+      <c r="E1732" t="inlineStr"/>
+      <c r="F1732" t="inlineStr">
+        <is>
+          <t>[H]O[C@]([H])(C(=O)N1C[C@H](Oc2cc(-c3ccccc3)nc3cc(OC)ccc23)C[C@H]1C(=O)N[C@]1(C(=O)NS(=O)(=O)C2CC2)C[C@@H]1CC)C1CCCCC1</t>
+        </is>
+      </c>
+      <c r="G1732" t="inlineStr"/>
+      <c r="H1732" t="inlineStr"/>
+      <c r="I1732" t="n">
+        <v>0.8964078813953507</v>
+      </c>
+      <c r="J1732" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1732" t="inlineStr"/>
+    </row>
+    <row r="1733">
+      <c r="A1733" s="1" t="n">
+        <v>1731</v>
+      </c>
+      <c r="B1733" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0072.png</t>
+        </is>
+      </c>
+      <c r="C1733" t="inlineStr"/>
+      <c r="D1733" t="inlineStr"/>
+      <c r="E1733" t="inlineStr"/>
+      <c r="F1733" t="inlineStr">
+        <is>
+          <t>O=C(NC(Cn1ccc(OCc2ccccc2)cc1=O)C(=O)N1CCC(N2CCCCC2)CC1)N1CCC(N2Cc3ccccc3NC2=O)CC1</t>
+        </is>
+      </c>
+      <c r="G1733" t="inlineStr"/>
+      <c r="H1733" t="inlineStr"/>
+      <c r="I1733" t="n">
+        <v>0.9173066312951518</v>
+      </c>
+      <c r="J1733" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1733" t="inlineStr"/>
+    </row>
+    <row r="1734">
+      <c r="A1734" s="1" t="n">
+        <v>1732</v>
+      </c>
+      <c r="B1734" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0073.png</t>
+        </is>
+      </c>
+      <c r="C1734" t="inlineStr"/>
+      <c r="D1734" t="inlineStr"/>
+      <c r="E1734" t="inlineStr"/>
+      <c r="F1734" t="inlineStr">
+        <is>
+          <t>c1ccc(-c2ccc(-c3ccccc3)c3c2-c2ccc4c5ccc6c7c(ccc(c8ccc-3c2c48)c75)-c2c(-c3ccccc3)ccc(-c3ccccc3)c2-6)cc1</t>
+        </is>
+      </c>
+      <c r="G1734" t="inlineStr"/>
+      <c r="H1734" t="inlineStr"/>
+      <c r="I1734" t="n">
+        <v>0.8780214396204282</v>
+      </c>
+      <c r="J1734" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1734" t="inlineStr"/>
+    </row>
+    <row r="1735">
+      <c r="A1735" s="1" t="n">
+        <v>1733</v>
+      </c>
+      <c r="B1735" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0074.png</t>
+        </is>
+      </c>
+      <c r="C1735" t="inlineStr"/>
+      <c r="D1735" t="inlineStr"/>
+      <c r="E1735" t="inlineStr"/>
+      <c r="F1735" t="inlineStr">
+        <is>
+          <t>c1ccc(-n2c(-c3cccc(-c4nc5c6ccccc6c6ccccc6c5n4-c4ccccc4)c3)nc3c4ccccc4c4ccccc4c32)cc1</t>
+        </is>
+      </c>
+      <c r="G1735" t="inlineStr"/>
+      <c r="H1735" t="inlineStr"/>
+      <c r="I1735" t="n">
+        <v>0.9079417429555183</v>
+      </c>
+      <c r="J1735" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1735" t="inlineStr"/>
+    </row>
+    <row r="1736">
+      <c r="A1736" s="1" t="n">
+        <v>1734</v>
+      </c>
+      <c r="B1736" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0075.png</t>
+        </is>
+      </c>
+      <c r="C1736" t="inlineStr"/>
+      <c r="D1736" t="inlineStr"/>
+      <c r="E1736" t="inlineStr"/>
+      <c r="F1736" t="inlineStr">
+        <is>
+          <t>CC1(C)O[C@@H]2[C@H](O1)[C@H](n1cnc3c(N)ncnc31)O[C@@H]2/C=C/CNC(=O)c1cc(C(=O)C2CCCCC2)cc2c1OC(c1ccccc1)(c1ccccc1)O2</t>
+        </is>
+      </c>
+      <c r="G1736" t="inlineStr"/>
+      <c r="H1736" t="inlineStr"/>
+      <c r="I1736" t="n">
+        <v>0.8940487163380083</v>
+      </c>
+      <c r="J1736" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1736" t="inlineStr"/>
+    </row>
+    <row r="1737">
+      <c r="A1737" s="1" t="n">
+        <v>1735</v>
+      </c>
+      <c r="B1737" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0076.png</t>
+        </is>
+      </c>
+      <c r="C1737" t="inlineStr"/>
+      <c r="D1737" t="inlineStr"/>
+      <c r="E1737" t="inlineStr"/>
+      <c r="F1737" t="inlineStr">
+        <is>
+          <t>CCN(CC)c1ccc(C(CC)(c2ccccc2)c2ccc(N(c3ccc(C)cc3)c3ccc4ccc5cccc6ccc3c4c56)cc2)cc1</t>
+        </is>
+      </c>
+      <c r="G1737" t="inlineStr"/>
+      <c r="H1737" t="inlineStr"/>
+      <c r="I1737" t="n">
+        <v>0.8823876040549724</v>
+      </c>
+      <c r="J1737" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1737" t="inlineStr"/>
+    </row>
+    <row r="1738">
+      <c r="A1738" s="1" t="n">
+        <v>1736</v>
+      </c>
+      <c r="B1738" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0077.png</t>
+        </is>
+      </c>
+      <c r="C1738" t="inlineStr"/>
+      <c r="D1738" t="inlineStr"/>
+      <c r="E1738" t="inlineStr"/>
+      <c r="F1738" t="inlineStr">
+        <is>
+          <t>Cc1cc(C)cc(-c2[nH]c3sc(C(C)(C)C(=O)N4C5CCC4CC5)cc3c2[C@H](C)CN/C(=N/C(=O)OC(C)C)N2CCN(CC(=O)NC(C)C)CC2)c1</t>
+        </is>
+      </c>
+      <c r="G1738" t="inlineStr"/>
+      <c r="H1738" t="inlineStr"/>
+      <c r="I1738" t="n">
+        <v>0.8852134504598471</v>
+      </c>
+      <c r="J1738" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1738" t="inlineStr"/>
+    </row>
+    <row r="1739">
+      <c r="A1739" s="1" t="n">
+        <v>1737</v>
+      </c>
+      <c r="B1739" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0078.png</t>
+        </is>
+      </c>
+      <c r="C1739" t="inlineStr"/>
+      <c r="D1739" t="inlineStr"/>
+      <c r="E1739" t="inlineStr"/>
+      <c r="F1739" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(cnn2CCCNC2=NCCCN2)c1)NS(=O)(=O)c1c(C)cc(OCCCC(=O)NCCNC(=O)C(CCC(=O)OC(C)(C)C)NC(=O)[C@@H](N)CCC(=O)OC(C)(C)C)cc1C</t>
+        </is>
+      </c>
+      <c r="G1739" t="inlineStr"/>
+      <c r="H1739" t="inlineStr"/>
+      <c r="I1739" t="n">
+        <v>0.8658121158163138</v>
+      </c>
+      <c r="J1739" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1739" t="inlineStr"/>
+    </row>
+    <row r="1740">
+      <c r="A1740" s="1" t="n">
+        <v>1738</v>
+      </c>
+      <c r="B1740" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0080.png</t>
+        </is>
+      </c>
+      <c r="C1740" t="inlineStr"/>
+      <c r="D1740" t="inlineStr"/>
+      <c r="E1740" t="inlineStr"/>
+      <c r="F1740" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(CNc3nccn3C(c3ccccc3)(c3ccccc3)c3ccccc3)nn(C)c2c1)NS(=O)(=O)c1ccc(-c2ccc(S(=O)(=O)NCCN)cc2)cc1</t>
+        </is>
+      </c>
+      <c r="G1740" t="inlineStr"/>
+      <c r="H1740" t="inlineStr"/>
+      <c r="I1740" t="n">
+        <v>0.8905611427299589</v>
+      </c>
+      <c r="J1740" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1740" t="inlineStr"/>
+    </row>
+    <row r="1741">
+      <c r="A1741" s="1" t="n">
+        <v>1739</v>
+      </c>
+      <c r="B1741" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0082.png</t>
+        </is>
+      </c>
+      <c r="C1741" t="inlineStr"/>
+      <c r="D1741" t="inlineStr"/>
+      <c r="E1741" t="inlineStr"/>
+      <c r="F1741" t="inlineStr">
+        <is>
+          <t>C=C[C@@H]1C[C@]1(NC(=O)[C@@H]1C[C@H](Oc2nc(-c3ccc(OC(F)(F)F)cc3)cc3cc(OC)ccc23)CN1C(=O)[C@@H](O)C(C)(C)C)C(=O)NS(=O)(=O)C1CC1</t>
+        </is>
+      </c>
+      <c r="G1741" t="inlineStr"/>
+      <c r="H1741" t="inlineStr"/>
+      <c r="I1741" t="n">
+        <v>0.8813345128149159</v>
+      </c>
+      <c r="J1741" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1741" t="inlineStr"/>
+    </row>
+    <row r="1742">
+      <c r="A1742" s="1" t="n">
+        <v>1740</v>
+      </c>
+      <c r="B1742" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0083.png</t>
+        </is>
+      </c>
+      <c r="C1742" t="inlineStr"/>
+      <c r="D1742" t="inlineStr"/>
+      <c r="E1742" t="inlineStr"/>
+      <c r="F1742" t="inlineStr">
+        <is>
+          <t>Cc1cc(C)cc(-c2[nH]c3sc(C(C)(C)C(=O)N4C5CCC4CC5)cc3c2[C@H](C)CN/C(=N/C(=O)OC(C)C)N2CCN(c3ccccn3)CC2)c1</t>
+        </is>
+      </c>
+      <c r="G1742" t="inlineStr"/>
+      <c r="H1742" t="inlineStr"/>
+      <c r="I1742" t="n">
+        <v>0.894047375489725</v>
+      </c>
+      <c r="J1742" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1742" t="inlineStr"/>
+    </row>
+    <row r="1743">
+      <c r="A1743" s="1" t="n">
+        <v>1741</v>
+      </c>
+      <c r="B1743" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0084.png</t>
+        </is>
+      </c>
+      <c r="C1743" t="inlineStr"/>
+      <c r="D1743" t="inlineStr"/>
+      <c r="E1743" t="inlineStr"/>
+      <c r="F1743" t="inlineStr">
+        <is>
+          <t>Cc1cc(OCCCC(=O)NCCNC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)OCc2ccccc2)cc(C)c1S(=O)(=O)N[C@@H](CNC(=O)c1ccc2c(cnn2CCNC2=NCCCC2)c1)C(=O)O</t>
+        </is>
+      </c>
+      <c r="G1743" t="inlineStr"/>
+      <c r="H1743" t="inlineStr"/>
+      <c r="I1743" t="n">
+        <v>0.8897775592653683</v>
+      </c>
+      <c r="J1743" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1743" t="inlineStr"/>
+    </row>
+    <row r="1744">
+      <c r="A1744" s="1" t="n">
+        <v>1742</v>
+      </c>
+      <c r="B1744" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0087.png</t>
+        </is>
+      </c>
+      <c r="C1744" t="inlineStr"/>
+      <c r="D1744" t="inlineStr"/>
+      <c r="E1744" t="inlineStr"/>
+      <c r="F1744" t="inlineStr">
+        <is>
+          <t>Cc1cc(C)cc(-c2[nH]c3sc(C(C)(C)C(=O)N4C5CCC4CC5)cc3c2[C@H](C)CN/C(=N/C(=O)OC(C)C)N2CCC(C3CCOCC3)CC2)c1</t>
+        </is>
+      </c>
+      <c r="G1744" t="inlineStr"/>
+      <c r="H1744" t="inlineStr"/>
+      <c r="I1744" t="n">
+        <v>0.9032333236516835</v>
+      </c>
+      <c r="J1744" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1744" t="inlineStr"/>
+    </row>
+    <row r="1745">
+      <c r="A1745" s="1" t="n">
+        <v>1743</v>
+      </c>
+      <c r="B1745" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0090.png</t>
+        </is>
+      </c>
+      <c r="C1745" t="inlineStr"/>
+      <c r="D1745" t="inlineStr"/>
+      <c r="E1745" t="inlineStr"/>
+      <c r="F1745" t="inlineStr">
+        <is>
+          <t>COC(=O)[C@H](CNC(=O)c1ccc2c(cnn2CCCNC2=NCCCN2)c1)NS(=O)(=O)c1ccc(-c2ccc(S(=O)(=O)NCCNC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)[C@H](CCC(=O)OC(C)(C)C)NC(=O)OCc3ccccc3)cc2)cc1</t>
+        </is>
+      </c>
+      <c r="G1745" t="inlineStr"/>
+      <c r="H1745" t="inlineStr"/>
+      <c r="I1745" t="n">
+        <v>0.8887643997989498</v>
+      </c>
+      <c r="J1745" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1745" t="inlineStr"/>
+    </row>
+    <row r="1746">
+      <c r="A1746" s="1" t="n">
+        <v>1744</v>
+      </c>
+      <c r="B1746" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0091.png</t>
+        </is>
+      </c>
+      <c r="C1746" t="inlineStr"/>
+      <c r="D1746" t="inlineStr"/>
+      <c r="E1746" t="inlineStr"/>
+      <c r="F1746" t="inlineStr">
+        <is>
+          <t>C=CCCCCCC(O)C(=O)N1C[C@H](Oc2nc(-c3ccccc3)cc3cc(OC)ccc23)CC1C(=O)N[C@]1(C(=O)NS(=O)(=O)C2CC2)C[C@H]1C=C</t>
+        </is>
+      </c>
+      <c r="G1746" t="inlineStr"/>
+      <c r="H1746" t="inlineStr"/>
+      <c r="I1746" t="n">
+        <v>0.9051356984152785</v>
+      </c>
+      <c r="J1746" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1746" t="inlineStr"/>
+    </row>
+    <row r="1747">
+      <c r="A1747" s="1" t="n">
+        <v>1745</v>
+      </c>
+      <c r="B1747" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0094.png</t>
+        </is>
+      </c>
+      <c r="C1747" t="inlineStr"/>
+      <c r="D1747" t="inlineStr"/>
+      <c r="E1747" t="inlineStr"/>
+      <c r="F1747" t="inlineStr">
+        <is>
+          <t>c1ccc2c(c1)-c1ccc(-c3ccc4ccc5cccnc5c4n3)cc1C21c2ccccc2-c2ccc(-c3ccc4ccc5cccnc5c4n3)cc21</t>
+        </is>
+      </c>
+      <c r="G1747" t="inlineStr"/>
+      <c r="H1747" t="inlineStr"/>
+      <c r="I1747" t="n">
+        <v>0.8941462661658132</v>
+      </c>
+      <c r="J1747" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1747" t="inlineStr"/>
+    </row>
+    <row r="1748">
+      <c r="A1748" s="1" t="n">
+        <v>1746</v>
+      </c>
+      <c r="B1748" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0097.png</t>
+        </is>
+      </c>
+      <c r="C1748" t="inlineStr"/>
+      <c r="D1748" t="inlineStr"/>
+      <c r="E1748" t="inlineStr"/>
+      <c r="F1748" t="inlineStr">
+        <is>
+          <t>CN(C)C(=O)c1cc2c(c(C(=O)NC/C=C/[C@H]3O[C@@H](n4cnc5c(N)ncnc54)[C@@H]4OC(C)(C)OC43)c1)OC(c1ccccc1)(c1ccccc1)O2</t>
+        </is>
+      </c>
+      <c r="G1748" t="inlineStr"/>
+      <c r="H1748" t="inlineStr"/>
+      <c r="I1748" t="n">
+        <v>0.9007253525525214</v>
+      </c>
+      <c r="J1748" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1748" t="inlineStr"/>
+    </row>
+    <row r="1749">
+      <c r="A1749" s="1" t="n">
+        <v>1747</v>
+      </c>
+      <c r="B1749" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0098.png</t>
+        </is>
+      </c>
+      <c r="C1749" t="inlineStr"/>
+      <c r="D1749" t="inlineStr"/>
+      <c r="E1749" t="inlineStr"/>
+      <c r="F1749" t="inlineStr">
+        <is>
+          <t>c1ccc2c(c1)-c1ccc(-c3ccc4ccc5ccccc5c4n3)cc1C21c2ccccc2-c2ccc(-c3ccc4ccc5ccccc5c4n3)cc21</t>
+        </is>
+      </c>
+      <c r="G1749" t="inlineStr"/>
+      <c r="H1749" t="inlineStr"/>
+      <c r="I1749" t="n">
+        <v>0.8852024857200894</v>
+      </c>
+      <c r="J1749" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1749" t="inlineStr"/>
+    </row>
+    <row r="1750">
+      <c r="A1750" s="1" t="n">
+        <v>1748</v>
+      </c>
+      <c r="B1750" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0099.png</t>
+        </is>
+      </c>
+      <c r="C1750" t="inlineStr"/>
+      <c r="D1750" t="inlineStr"/>
+      <c r="E1750" t="inlineStr"/>
+      <c r="F1750" t="inlineStr">
+        <is>
+          <t>CCc1ccc(-c2ccc(CN(C)c3ccc(-c4cccc(-c5ccc(N(C)Cc6ccc(-c7ccc(C)cc7)cc6)cc5)c4)cc3)cc2)cc1</t>
+        </is>
+      </c>
+      <c r="G1750" t="inlineStr"/>
+      <c r="H1750" t="inlineStr"/>
+      <c r="I1750" t="n">
+        <v>0.8692438665110074</v>
+      </c>
+      <c r="J1750" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1750" t="inlineStr"/>
+    </row>
+    <row r="1751">
+      <c r="A1751" s="1" t="n">
+        <v>1749</v>
+      </c>
+      <c r="B1751" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T061928/rb_0100.png</t>
+        </is>
+      </c>
+      <c r="C1751" t="inlineStr"/>
+      <c r="D1751" t="inlineStr"/>
+      <c r="E1751" t="inlineStr"/>
+      <c r="F1751" t="inlineStr">
+        <is>
+          <t>[H][C@@](NC(=O)N(C)Cc1csc(C(C)C)n1)(C(=O)N[C@@](C)(Cc1ccccc1)C[C@H](O)[C@]([H])(Cc1ccccc1)NC(=O)OCc1cncs1)C(C)C</t>
+        </is>
+      </c>
+      <c r="G1751" t="inlineStr"/>
+      <c r="H1751" t="inlineStr"/>
+      <c r="I1751" t="n">
+        <v>0.8913209820059446</v>
+      </c>
+      <c r="J1751" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1751" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Superatoms big set: +250 drawings, 250 API reads, 250 CXMolScribe reads
C-MAGE big superatoms: +250 drawings ({'macrocycle': 96, 'peptide': 35, 'protac': 119}), 250 read by Sonnet 5.5 API ($9.35), 250 by CXMolScribe; 350 read in all, PROTACs 119/3000; big-set API $11.99/140.
Exact: USPTO: API 63/100 63.0%, CX 54/100 54.0%; USPTO-ODP: API 191/250 76.4%, CX 135/250 54.0%

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/published_runs/sonnet55_api_superatoms/cxmolscribe/Completed_HighConfidence_CMAGE.xlsx
+++ b/benchmarks/published_runs/sonnet55_api_superatoms/cxmolscribe/Completed_HighConfidence_CMAGE.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1751"/>
+  <dimension ref="A1:K1906"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51230,6 +51230,4501 @@
       </c>
       <c r="K1751" t="inlineStr"/>
     </row>
+    <row r="1752">
+      <c r="A1752" s="1" t="n">
+        <v>1750</v>
+      </c>
+      <c r="B1752" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0101.png</t>
+        </is>
+      </c>
+      <c r="C1752" t="inlineStr"/>
+      <c r="D1752" t="inlineStr"/>
+      <c r="E1752" t="inlineStr"/>
+      <c r="F1752" t="inlineStr">
+        <is>
+          <t>Cc1[nH]c2ccccc2c1C[C@H]1C(=O)NCc2c(-c3ccn(CC(=O)O)c(=O)c3)ccc(Cl)c2Sc2ncccc2CN[C@@H](CCCN)C(=O)N[C@@H](CCCCN)C(=O)N1C</t>
+        </is>
+      </c>
+      <c r="G1752" t="inlineStr"/>
+      <c r="H1752" t="inlineStr"/>
+      <c r="I1752" t="n">
+        <v>0.890906805239708</v>
+      </c>
+      <c r="J1752" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1752" t="inlineStr"/>
+    </row>
+    <row r="1753">
+      <c r="A1753" s="1" t="n">
+        <v>1751</v>
+      </c>
+      <c r="B1753" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0102.png</t>
+        </is>
+      </c>
+      <c r="C1753" t="inlineStr"/>
+      <c r="D1753" t="inlineStr"/>
+      <c r="E1753" t="inlineStr"/>
+      <c r="F1753" t="inlineStr">
+        <is>
+          <t>CC(C)(S)[C@H](NC(=O)[C@H](CC(=O)O)NC(=O)[C@H](CCCCN)NC(=O)[C@H](CC(=O)O)NC(=O)CCC(=O)Nc1cccc2c(C(=O)NCC(=O)N3CC(F)(F)C[C@H]3C#N)ccnc12)C(=O)O</t>
+        </is>
+      </c>
+      <c r="G1753" t="inlineStr"/>
+      <c r="H1753" t="inlineStr"/>
+      <c r="I1753" t="n">
+        <v>0.8890425487913143</v>
+      </c>
+      <c r="J1753" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1753" t="inlineStr"/>
+    </row>
+    <row r="1754">
+      <c r="A1754" s="1" t="n">
+        <v>1752</v>
+      </c>
+      <c r="B1754" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0105.png</t>
+        </is>
+      </c>
+      <c r="C1754" t="inlineStr"/>
+      <c r="D1754" t="inlineStr"/>
+      <c r="E1754" t="inlineStr"/>
+      <c r="F1754" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4ccc(CN[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)cc4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1754" t="inlineStr"/>
+      <c r="H1754" t="inlineStr"/>
+      <c r="I1754" t="n">
+        <v>0.8887266634880251</v>
+      </c>
+      <c r="J1754" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1754" t="inlineStr"/>
+    </row>
+    <row r="1755">
+      <c r="A1755" s="1" t="n">
+        <v>1753</v>
+      </c>
+      <c r="B1755" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0106.png</t>
+        </is>
+      </c>
+      <c r="C1755" t="inlineStr"/>
+      <c r="D1755" t="inlineStr"/>
+      <c r="E1755" t="inlineStr"/>
+      <c r="F1755" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)CCC(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1755" t="inlineStr"/>
+      <c r="H1755" t="inlineStr"/>
+      <c r="I1755" t="n">
+        <v>0.8928162500331304</v>
+      </c>
+      <c r="J1755" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1755" t="inlineStr"/>
+    </row>
+    <row r="1756">
+      <c r="A1756" s="1" t="n">
+        <v>1754</v>
+      </c>
+      <c r="B1756" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0107.png</t>
+        </is>
+      </c>
+      <c r="C1756" t="inlineStr"/>
+      <c r="D1756" t="inlineStr"/>
+      <c r="E1756" t="inlineStr"/>
+      <c r="F1756" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)[C@@H]4C[C@@H](C(=O)N[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)C4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1756" t="inlineStr"/>
+      <c r="H1756" t="inlineStr"/>
+      <c r="I1756" t="n">
+        <v>0.9035510515789659</v>
+      </c>
+      <c r="J1756" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1756" t="inlineStr"/>
+    </row>
+    <row r="1757">
+      <c r="A1757" s="1" t="n">
+        <v>1755</v>
+      </c>
+      <c r="B1757" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0108.png</t>
+        </is>
+      </c>
+      <c r="C1757" t="inlineStr"/>
+      <c r="D1757" t="inlineStr"/>
+      <c r="E1757" t="inlineStr"/>
+      <c r="F1757" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2ccc(C3=C4C=c5ccccc5=[N+]4[B-](F)(F)n4c3cc3ccccc34)cc2OC)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1757" t="inlineStr"/>
+      <c r="H1757" t="inlineStr"/>
+      <c r="I1757" t="n">
+        <v>0.9050060473668353</v>
+      </c>
+      <c r="J1757" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1757" t="inlineStr"/>
+    </row>
+    <row r="1758">
+      <c r="A1758" s="1" t="n">
+        <v>1756</v>
+      </c>
+      <c r="B1758" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0109.png</t>
+        </is>
+      </c>
+      <c r="C1758" t="inlineStr"/>
+      <c r="D1758" t="inlineStr"/>
+      <c r="E1758" t="inlineStr"/>
+      <c r="F1758" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN7CC8CCC7C8)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1758" t="inlineStr"/>
+      <c r="H1758" t="inlineStr"/>
+      <c r="I1758" t="n">
+        <v>0.8876300268363819</v>
+      </c>
+      <c r="J1758" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1758" t="inlineStr"/>
+    </row>
+    <row r="1759">
+      <c r="A1759" s="1" t="n">
+        <v>1757</v>
+      </c>
+      <c r="B1759" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0110.png</t>
+        </is>
+      </c>
+      <c r="C1759" t="inlineStr"/>
+      <c r="D1759" t="inlineStr"/>
+      <c r="E1759" t="inlineStr"/>
+      <c r="F1759" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4ccc(C(=O)N[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)cc4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1759" t="inlineStr"/>
+      <c r="H1759" t="inlineStr"/>
+      <c r="I1759" t="n">
+        <v>0.9027908563676383</v>
+      </c>
+      <c r="J1759" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1759" t="inlineStr"/>
+    </row>
+    <row r="1760">
+      <c r="A1760" s="1" t="n">
+        <v>1758</v>
+      </c>
+      <c r="B1760" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0111.png</t>
+        </is>
+      </c>
+      <c r="C1760" t="inlineStr"/>
+      <c r="D1760" t="inlineStr"/>
+      <c r="E1760" t="inlineStr"/>
+      <c r="F1760" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc([C@H](C)NC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)c2ccc(N3CCN(c4cc(-c5ccccc5O)nnc4N)CC3)s2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1760" t="inlineStr"/>
+      <c r="H1760" t="inlineStr"/>
+      <c r="I1760" t="n">
+        <v>0.8918146782755171</v>
+      </c>
+      <c r="J1760" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1760" t="inlineStr"/>
+    </row>
+    <row r="1761">
+      <c r="A1761" s="1" t="n">
+        <v>1759</v>
+      </c>
+      <c r="B1761" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0112.png</t>
+        </is>
+      </c>
+      <c r="C1761" t="inlineStr"/>
+      <c r="D1761" t="inlineStr"/>
+      <c r="E1761" t="inlineStr"/>
+      <c r="F1761" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc(CNC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)N(CCCCNC[C@@H]2CC[C@@H](n3cc4cc(NC(=O)c5cccc(C(F)(F)F)n5)c(C(C)(C)O)cc4n3)CC2)CCCCN2CCC(c3ccc(Nc4nc(N5CCCCC5)cnc4C(N)=O)cc3)CC2)C(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1761" t="inlineStr"/>
+      <c r="H1761" t="inlineStr"/>
+      <c r="I1761" t="n">
+        <v>0.8835469944379127</v>
+      </c>
+      <c r="J1761" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1761" t="inlineStr"/>
+    </row>
+    <row r="1762">
+      <c r="A1762" s="1" t="n">
+        <v>1760</v>
+      </c>
+      <c r="B1762" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0114.png</t>
+        </is>
+      </c>
+      <c r="C1762" t="inlineStr"/>
+      <c r="D1762" t="inlineStr"/>
+      <c r="E1762" t="inlineStr"/>
+      <c r="F1762" t="inlineStr">
+        <is>
+          <t>N[C@@H](Cc1ccc(NS(=O)(=O)c2ccc(C3CCCCC3)cc2)cc1)C(=O)N1CCC(CCC#Cc2cccc3c2CN(C2CCC(=O)NC2=O)C3=O)CC1</t>
+        </is>
+      </c>
+      <c r="G1762" t="inlineStr"/>
+      <c r="H1762" t="inlineStr"/>
+      <c r="I1762" t="n">
+        <v>0.9037736828754294</v>
+      </c>
+      <c r="J1762" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1762" t="inlineStr"/>
+    </row>
+    <row r="1763">
+      <c r="A1763" s="1" t="n">
+        <v>1761</v>
+      </c>
+      <c r="B1763" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0116.png</t>
+        </is>
+      </c>
+      <c r="C1763" t="inlineStr"/>
+      <c r="D1763" t="inlineStr"/>
+      <c r="E1763" t="inlineStr"/>
+      <c r="F1763" t="inlineStr">
+        <is>
+          <t>CCOP(=O)(O)C(F)(F)c1ccc2[nH]c(C(=O)N[C@H]3CN(CCOCCOCCOCCNc4cccc5c4C(=O)N(C4CCC(=O)NC4=O)C5=O)CC[C@H]4CC[C@@H](C(=O)NCCCC(N)=O)N4C3=O)cc2c1</t>
+        </is>
+      </c>
+      <c r="G1763" t="inlineStr"/>
+      <c r="H1763" t="inlineStr"/>
+      <c r="I1763" t="n">
+        <v>0.8793957597443802</v>
+      </c>
+      <c r="J1763" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1763" t="inlineStr"/>
+    </row>
+    <row r="1764">
+      <c r="A1764" s="1" t="n">
+        <v>1762</v>
+      </c>
+      <c r="B1764" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0117.png</t>
+        </is>
+      </c>
+      <c r="C1764" t="inlineStr"/>
+      <c r="D1764" t="inlineStr"/>
+      <c r="E1764" t="inlineStr"/>
+      <c r="F1764" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)CCC(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1764" t="inlineStr"/>
+      <c r="H1764" t="inlineStr"/>
+      <c r="I1764" t="n">
+        <v>0.8875698715321245</v>
+      </c>
+      <c r="J1764" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1764" t="inlineStr"/>
+    </row>
+    <row r="1765">
+      <c r="A1765" s="1" t="n">
+        <v>1763</v>
+      </c>
+      <c r="B1765" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0118.png</t>
+        </is>
+      </c>
+      <c r="C1765" t="inlineStr"/>
+      <c r="D1765" t="inlineStr"/>
+      <c r="E1765" t="inlineStr"/>
+      <c r="F1765" t="inlineStr">
+        <is>
+          <t>C#C[Br-]1(C#C)N2C(C)=CC(C)=C2C(C2=CC=C(N3CCOCCOCCN(C4=C(OC)C=CC=C4)CCOCCOCC3)C(OC)=C2)=C2C(C)=CC(C)=[N+]21</t>
+        </is>
+      </c>
+      <c r="G1765" t="inlineStr"/>
+      <c r="H1765" t="inlineStr"/>
+      <c r="I1765" t="n">
+        <v>0.8863642561670542</v>
+      </c>
+      <c r="J1765" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1765" t="inlineStr"/>
+    </row>
+    <row r="1766">
+      <c r="A1766" s="1" t="n">
+        <v>1764</v>
+      </c>
+      <c r="B1766" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0119.png</t>
+        </is>
+      </c>
+      <c r="C1766" t="inlineStr"/>
+      <c r="D1766" t="inlineStr"/>
+      <c r="E1766" t="inlineStr"/>
+      <c r="F1766" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4cc(C(=O)N[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)ncn4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1766" t="inlineStr"/>
+      <c r="H1766" t="inlineStr"/>
+      <c r="I1766" t="n">
+        <v>0.8823817498528365</v>
+      </c>
+      <c r="J1766" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1766" t="inlineStr"/>
+    </row>
+    <row r="1767">
+      <c r="A1767" s="1" t="n">
+        <v>1765</v>
+      </c>
+      <c r="B1767" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0121.png</t>
+        </is>
+      </c>
+      <c r="C1767" t="inlineStr"/>
+      <c r="D1767" t="inlineStr"/>
+      <c r="E1767" t="inlineStr"/>
+      <c r="F1767" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCN(c2cc(C3=C4C=CC(=[N+](C)C)C=C4C(C)(C)c4cc(N(C)C)ccc43)c(C(=O)[O-])cc2OC)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1767" t="inlineStr"/>
+      <c r="H1767" t="inlineStr"/>
+      <c r="I1767" t="n">
+        <v>0.8940898481672558</v>
+      </c>
+      <c r="J1767" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1767" t="inlineStr"/>
+    </row>
+    <row r="1768">
+      <c r="A1768" s="1" t="n">
+        <v>1766</v>
+      </c>
+      <c r="B1768" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0122.png</t>
+        </is>
+      </c>
+      <c r="C1768" t="inlineStr"/>
+      <c r="D1768" t="inlineStr"/>
+      <c r="E1768" t="inlineStr"/>
+      <c r="F1768" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2cc3c(cc2OC)C2(OC3=O)c3ccc(OC(C)=O)cc3S(=O)(=O)c3cc(OC(C)=O)ccc32)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1768" t="inlineStr"/>
+      <c r="H1768" t="inlineStr"/>
+      <c r="I1768" t="n">
+        <v>0.9000330186341481</v>
+      </c>
+      <c r="J1768" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1768" t="inlineStr"/>
+    </row>
+    <row r="1769">
+      <c r="A1769" s="1" t="n">
+        <v>1767</v>
+      </c>
+      <c r="B1769" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0123.png</t>
+        </is>
+      </c>
+      <c r="C1769" t="inlineStr"/>
+      <c r="D1769" t="inlineStr"/>
+      <c r="E1769" t="inlineStr"/>
+      <c r="F1769" t="inlineStr">
+        <is>
+          <t>O=C(O)c1cccc(CN2CCOCCOCCN(Cc3cc(OCCc4ccc(N=C=S)cc4)cc(C(=O)O)n3)CCOCCOCC2)n1</t>
+        </is>
+      </c>
+      <c r="G1769" t="inlineStr"/>
+      <c r="H1769" t="inlineStr"/>
+      <c r="I1769" t="n">
+        <v>0.8437937674634005</v>
+      </c>
+      <c r="J1769" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1769" t="inlineStr"/>
+    </row>
+    <row r="1770">
+      <c r="A1770" s="1" t="n">
+        <v>1768</v>
+      </c>
+      <c r="B1770" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0126.png</t>
+        </is>
+      </c>
+      <c r="C1770" t="inlineStr"/>
+      <c r="D1770" t="inlineStr"/>
+      <c r="E1770" t="inlineStr"/>
+      <c r="F1770" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN7CCCCCC7)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1770" t="inlineStr"/>
+      <c r="H1770" t="inlineStr"/>
+      <c r="I1770" t="n">
+        <v>0.8881306513092286</v>
+      </c>
+      <c r="J1770" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1770" t="inlineStr"/>
+    </row>
+    <row r="1771">
+      <c r="A1771" s="1" t="n">
+        <v>1769</v>
+      </c>
+      <c r="B1771" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0127.png</t>
+        </is>
+      </c>
+      <c r="C1771" t="inlineStr"/>
+      <c r="D1771" t="inlineStr"/>
+      <c r="E1771" t="inlineStr"/>
+      <c r="F1771" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc([C@H](C)NC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)CN2CCN(c3cc(-c4cccc(F)c4O)nnc3N)CC2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1771" t="inlineStr"/>
+      <c r="H1771" t="inlineStr"/>
+      <c r="I1771" t="n">
+        <v>0.8992640380749422</v>
+      </c>
+      <c r="J1771" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1771" t="inlineStr"/>
+    </row>
+    <row r="1772">
+      <c r="A1772" s="1" t="n">
+        <v>1770</v>
+      </c>
+      <c r="B1772" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0129.png</t>
+        </is>
+      </c>
+      <c r="C1772" t="inlineStr"/>
+      <c r="D1772" t="inlineStr"/>
+      <c r="E1772" t="inlineStr"/>
+      <c r="F1772" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2cc(C(=O)O)c(C3=C4C=C(F)C(=O)C=C4B(O)c4cc(O)c(F)cc43)cc2OC)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1772" t="inlineStr"/>
+      <c r="H1772" t="inlineStr"/>
+      <c r="I1772" t="n">
+        <v>0.9087582354940286</v>
+      </c>
+      <c r="J1772" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1772" t="inlineStr"/>
+    </row>
+    <row r="1773">
+      <c r="A1773" s="1" t="n">
+        <v>1771</v>
+      </c>
+      <c r="B1773" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0131.png</t>
+        </is>
+      </c>
+      <c r="C1773" t="inlineStr"/>
+      <c r="D1773" t="inlineStr"/>
+      <c r="E1773" t="inlineStr"/>
+      <c r="F1773" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2cc3c(cc2OC)C2(OC3=O)c3ccc(OC(C)=O)cc3P(C)(=O)c3cc(OC(C)=O)ccc32)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1773" t="inlineStr"/>
+      <c r="H1773" t="inlineStr"/>
+      <c r="I1773" t="n">
+        <v>0.9031096149582338</v>
+      </c>
+      <c r="J1773" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1773" t="inlineStr"/>
+    </row>
+    <row r="1774">
+      <c r="A1774" s="1" t="n">
+        <v>1772</v>
+      </c>
+      <c r="B1774" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0133.png</t>
+        </is>
+      </c>
+      <c r="C1774" t="inlineStr"/>
+      <c r="D1774" t="inlineStr"/>
+      <c r="E1774" t="inlineStr"/>
+      <c r="F1774" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2ccc(C3=C4C(C)=CC(C)=[N+]4[B-](OC)(OC)n4c(C)cc(C)c43)cc2OC)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1774" t="inlineStr"/>
+      <c r="H1774" t="inlineStr"/>
+      <c r="I1774" t="n">
+        <v>0.9067113547843993</v>
+      </c>
+      <c r="J1774" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1774" t="inlineStr"/>
+    </row>
+    <row r="1775">
+      <c r="A1775" s="1" t="n">
+        <v>1773</v>
+      </c>
+      <c r="B1775" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0135.png</t>
+        </is>
+      </c>
+      <c r="C1775" t="inlineStr"/>
+      <c r="D1775" t="inlineStr"/>
+      <c r="E1775" t="inlineStr"/>
+      <c r="F1775" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccc2c(c1)CCCOc1cc(ccc1Cc1nc3c(OCCOC)cc(C(=O)OC)cc3n1C[C@@H]1CCO1)-c1cccc(n1)OC2</t>
+        </is>
+      </c>
+      <c r="G1775" t="inlineStr"/>
+      <c r="H1775" t="inlineStr"/>
+      <c r="I1775" t="n">
+        <v>0.8796212786983971</v>
+      </c>
+      <c r="J1775" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1775" t="inlineStr"/>
+    </row>
+    <row r="1776">
+      <c r="A1776" s="1" t="n">
+        <v>1774</v>
+      </c>
+      <c r="B1776" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0138.png</t>
+        </is>
+      </c>
+      <c r="C1776" t="inlineStr"/>
+      <c r="D1776" t="inlineStr"/>
+      <c r="E1776" t="inlineStr"/>
+      <c r="F1776" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2cc3c(cc2OC)C2(OC3=O)c3ccc(OC(C)=O)cc3[Si](C)(C)c3cc(OC(C)=O)ccc32)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1776" t="inlineStr"/>
+      <c r="H1776" t="inlineStr"/>
+      <c r="I1776" t="n">
+        <v>0.9029322857220686</v>
+      </c>
+      <c r="J1776" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1776" t="inlineStr"/>
+    </row>
+    <row r="1777">
+      <c r="A1777" s="1" t="n">
+        <v>1775</v>
+      </c>
+      <c r="B1777" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0141.png</t>
+        </is>
+      </c>
+      <c r="C1777" t="inlineStr"/>
+      <c r="D1777" t="inlineStr"/>
+      <c r="E1777" t="inlineStr"/>
+      <c r="F1777" t="inlineStr">
+        <is>
+          <t>Cc1cnc(Nc2cc(C3CCN(C(=O)C4CC(C(=O)Nc5cccc6c5C(=O)N(C5CCC(=O)NC5=O)C6=O)C4)CC3)cc(N3CCC(F)(F)C3)n2)cn1</t>
+        </is>
+      </c>
+      <c r="G1777" t="inlineStr"/>
+      <c r="H1777" t="inlineStr"/>
+      <c r="I1777" t="n">
+        <v>0.888462048485224</v>
+      </c>
+      <c r="J1777" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1777" t="inlineStr"/>
+    </row>
+    <row r="1778">
+      <c r="A1778" s="1" t="n">
+        <v>1776</v>
+      </c>
+      <c r="B1778" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0142.png</t>
+        </is>
+      </c>
+      <c r="C1778" t="inlineStr"/>
+      <c r="D1778" t="inlineStr"/>
+      <c r="E1778" t="inlineStr"/>
+      <c r="F1778" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc(CNC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)CCCCCCCCCCCOc2ccc3c(-c4ccc(C(=O)O)c(C5CCCC5)c4)ncnc3c2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1778" t="inlineStr"/>
+      <c r="H1778" t="inlineStr"/>
+      <c r="I1778" t="n">
+        <v>0.8798559839417448</v>
+      </c>
+      <c r="J1778" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1778" t="inlineStr"/>
+    </row>
+    <row r="1779">
+      <c r="A1779" s="1" t="n">
+        <v>1777</v>
+      </c>
+      <c r="B1779" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0144.png</t>
+        </is>
+      </c>
+      <c r="C1779" t="inlineStr"/>
+      <c r="D1779" t="inlineStr"/>
+      <c r="E1779" t="inlineStr"/>
+      <c r="F1779" t="inlineStr">
+        <is>
+          <t>NC(=O)c1c(-c2ccc(Oc3ccccc3)cc2)nn2c1Nc1ccc(NCC3CCN(c4ccc5c(c4)C(=O)N(C4CCC(=O)NC4=O)C5=O)CC3)cc1CC2</t>
+        </is>
+      </c>
+      <c r="G1779" t="inlineStr"/>
+      <c r="H1779" t="inlineStr"/>
+      <c r="I1779" t="n">
+        <v>0.8864810231225339</v>
+      </c>
+      <c r="J1779" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1779" t="inlineStr"/>
+    </row>
+    <row r="1780">
+      <c r="A1780" s="1" t="n">
+        <v>1778</v>
+      </c>
+      <c r="B1780" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0145.png</t>
+        </is>
+      </c>
+      <c r="C1780" t="inlineStr"/>
+      <c r="D1780" t="inlineStr"/>
+      <c r="E1780" t="inlineStr"/>
+      <c r="F1780" t="inlineStr">
+        <is>
+          <t>COCCOc1cc(C(=O)O)cc2c1nc(Cc1cc(F)c3cc1COCCc1cc(C#N)cc(F)c1COc1cccc-3n1)n2C[C@@H]1CCO1</t>
+        </is>
+      </c>
+      <c r="G1780" t="inlineStr"/>
+      <c r="H1780" t="inlineStr"/>
+      <c r="I1780" t="n">
+        <v>0.898045312028382</v>
+      </c>
+      <c r="J1780" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1780" t="inlineStr"/>
+    </row>
+    <row r="1781">
+      <c r="A1781" s="1" t="n">
+        <v>1779</v>
+      </c>
+      <c r="B1781" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0146.png</t>
+        </is>
+      </c>
+      <c r="C1781" t="inlineStr"/>
+      <c r="D1781" t="inlineStr"/>
+      <c r="E1781" t="inlineStr"/>
+      <c r="F1781" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCCN)NC(=O)[C@H](CCCN)NCc2nccnc2Sc2c(Cl)ccc(-c3ccc(C(=O)O)cc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1781" t="inlineStr"/>
+      <c r="H1781" t="inlineStr"/>
+      <c r="I1781" t="n">
+        <v>0.8907545307378212</v>
+      </c>
+      <c r="J1781" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1781" t="inlineStr"/>
+    </row>
+    <row r="1782">
+      <c r="A1782" s="1" t="n">
+        <v>1780</v>
+      </c>
+      <c r="B1782" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0149.png</t>
+        </is>
+      </c>
+      <c r="C1782" t="inlineStr"/>
+      <c r="D1782" t="inlineStr"/>
+      <c r="E1782" t="inlineStr"/>
+      <c r="F1782" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(O)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1782" t="inlineStr"/>
+      <c r="H1782" t="inlineStr"/>
+      <c r="I1782" t="n">
+        <v>0.8762769975916448</v>
+      </c>
+      <c r="J1782" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1782" t="inlineStr"/>
+    </row>
+    <row r="1783">
+      <c r="A1783" s="1" t="n">
+        <v>1781</v>
+      </c>
+      <c r="B1783" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0150.png</t>
+        </is>
+      </c>
+      <c r="C1783" t="inlineStr"/>
+      <c r="D1783" t="inlineStr"/>
+      <c r="E1783" t="inlineStr"/>
+      <c r="F1783" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc([C@H](C)NC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)[C@@H]2C[C@@H](C(=O)N3CCC(c4cc(Nc5cnccn5)nc(N5CCC(F)(F)C5)c4)CC3)C2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1783" t="inlineStr"/>
+      <c r="H1783" t="inlineStr"/>
+      <c r="I1783" t="n">
+        <v>0.8978856498306861</v>
+      </c>
+      <c r="J1783" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1783" t="inlineStr"/>
+    </row>
+    <row r="1784">
+      <c r="A1784" s="1" t="n">
+        <v>1782</v>
+      </c>
+      <c r="B1784" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0151.png</t>
+        </is>
+      </c>
+      <c r="C1784" t="inlineStr"/>
+      <c r="D1784" t="inlineStr"/>
+      <c r="E1784" t="inlineStr"/>
+      <c r="F1784" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCN)NC(=O)[C@H](CCN)NCc2cccnc2Sc2c(Cl)ccc(-c3ccc(C(=O)O)cc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1784" t="inlineStr"/>
+      <c r="H1784" t="inlineStr"/>
+      <c r="I1784" t="n">
+        <v>0.8987201279751899</v>
+      </c>
+      <c r="J1784" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1784" t="inlineStr"/>
+    </row>
+    <row r="1785">
+      <c r="A1785" s="1" t="n">
+        <v>1783</v>
+      </c>
+      <c r="B1785" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0152.png</t>
+        </is>
+      </c>
+      <c r="C1785" t="inlineStr"/>
+      <c r="D1785" t="inlineStr"/>
+      <c r="E1785" t="inlineStr"/>
+      <c r="F1785" t="inlineStr">
+        <is>
+          <t>CC[C@@]1(O)C(=O)OCc2c1cc1n(c2=O)Cc2c-1nc1cc(F)c(C)cc1c2CCCCOCNC(=O)[C@H](C)NC(=O)[C@H](C)NC(=O)[C@H](C)NC(=O)[C@H](CCC(=O)N(C)C[C@H](O)[C@@H](O)[C@H](O)[C@H](O)CO)NC(=O)CCN1C(=O)C=CC1=O</t>
+        </is>
+      </c>
+      <c r="G1785" t="inlineStr"/>
+      <c r="H1785" t="inlineStr"/>
+      <c r="I1785" t="n">
+        <v>0.8844931128978811</v>
+      </c>
+      <c r="J1785" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1785" t="inlineStr"/>
+    </row>
+    <row r="1786">
+      <c r="A1786" s="1" t="n">
+        <v>1784</v>
+      </c>
+      <c r="B1786" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0157.png</t>
+        </is>
+      </c>
+      <c r="C1786" t="inlineStr"/>
+      <c r="D1786" t="inlineStr"/>
+      <c r="E1786" t="inlineStr"/>
+      <c r="F1786" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4ccc(-c5ccc(C(=O)N[C@H](C(=O)N6C[C@H](O)C[C@H]6C(=O)N[C@@H](C)c6ccc(-c7scnc7C)cc6)C(C)(C)C)cc5)cc4)C3C)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1786" t="inlineStr"/>
+      <c r="H1786" t="inlineStr"/>
+      <c r="I1786" t="n">
+        <v>0.8559881206764496</v>
+      </c>
+      <c r="J1786" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1786" t="inlineStr"/>
+    </row>
+    <row r="1787">
+      <c r="A1787" s="1" t="n">
+        <v>1785</v>
+      </c>
+      <c r="B1787" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0159.png</t>
+        </is>
+      </c>
+      <c r="C1787" t="inlineStr"/>
+      <c r="D1787" t="inlineStr"/>
+      <c r="E1787" t="inlineStr"/>
+      <c r="F1787" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)CCCCCN[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1787" t="inlineStr"/>
+      <c r="H1787" t="inlineStr"/>
+      <c r="I1787" t="n">
+        <v>0.8849592370387845</v>
+      </c>
+      <c r="J1787" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1787" t="inlineStr"/>
+    </row>
+    <row r="1788">
+      <c r="A1788" s="1" t="n">
+        <v>1786</v>
+      </c>
+      <c r="B1788" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0165.png</t>
+        </is>
+      </c>
+      <c r="C1788" t="inlineStr"/>
+      <c r="D1788" t="inlineStr"/>
+      <c r="E1788" t="inlineStr"/>
+      <c r="F1788" t="inlineStr">
+        <is>
+          <t>COC(=O)c1cc(NC[C@@H]2CCO2)c(NC(=O)Cc2ccc3cc2COCCc2cc(Cl)ccc2COc2cccc-3n2)c(OCCO[Si](C)(C)C(C)(C)C)c1</t>
+        </is>
+      </c>
+      <c r="G1788" t="inlineStr"/>
+      <c r="H1788" t="inlineStr"/>
+      <c r="I1788" t="n">
+        <v>0.894287291088156</v>
+      </c>
+      <c r="J1788" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1788" t="inlineStr"/>
+    </row>
+    <row r="1789">
+      <c r="A1789" s="1" t="n">
+        <v>1787</v>
+      </c>
+      <c r="B1789" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0166.png</t>
+        </is>
+      </c>
+      <c r="C1789" t="inlineStr"/>
+      <c r="D1789" t="inlineStr"/>
+      <c r="E1789" t="inlineStr"/>
+      <c r="F1789" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCNC(=O)OC(C)(C)C)NC(=O)[C@H](CCCNC(=O)OC(C)(C)C)NCc2cccnc2Sc2c(F)ccc(Br)c2CNC(=O)[C@@H]1Cc1cn(C(=O)OC(C)(C)C)c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1789" t="inlineStr"/>
+      <c r="H1789" t="inlineStr"/>
+      <c r="I1789" t="n">
+        <v>0.9065416330662514</v>
+      </c>
+      <c r="J1789" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1789" t="inlineStr"/>
+    </row>
+    <row r="1790">
+      <c r="A1790" s="1" t="n">
+        <v>1788</v>
+      </c>
+      <c r="B1790" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0167.png</t>
+        </is>
+      </c>
+      <c r="C1790" t="inlineStr"/>
+      <c r="D1790" t="inlineStr"/>
+      <c r="E1790" t="inlineStr"/>
+      <c r="F1790" t="inlineStr">
+        <is>
+          <t>CC(C)c1cnn2c(NCc3ccccc3-c3nccc4cc(NCC5CCN(CC6CCN(c7ccc8c(c7)C(=O)N(C7CCC(=O)NC7=O)C8=O)CC6)CC5)ccc34)nc(N[C@@H]3CCCNC3)nc12</t>
+        </is>
+      </c>
+      <c r="G1790" t="inlineStr"/>
+      <c r="H1790" t="inlineStr"/>
+      <c r="I1790" t="n">
+        <v>0.8975483277394064</v>
+      </c>
+      <c r="J1790" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1790" t="inlineStr"/>
+    </row>
+    <row r="1791">
+      <c r="A1791" s="1" t="n">
+        <v>1789</v>
+      </c>
+      <c r="B1791" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0168.png</t>
+        </is>
+      </c>
+      <c r="C1791" t="inlineStr"/>
+      <c r="D1791" t="inlineStr"/>
+      <c r="E1791" t="inlineStr"/>
+      <c r="F1791" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN(C)c7ccccn7)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1791" t="inlineStr"/>
+      <c r="H1791" t="inlineStr"/>
+      <c r="I1791" t="n">
+        <v>0.8929740635843338</v>
+      </c>
+      <c r="J1791" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1791" t="inlineStr"/>
+    </row>
+    <row r="1792">
+      <c r="A1792" s="1" t="n">
+        <v>1790</v>
+      </c>
+      <c r="B1792" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0169.png</t>
+        </is>
+      </c>
+      <c r="C1792" t="inlineStr"/>
+      <c r="D1792" t="inlineStr"/>
+      <c r="E1792" t="inlineStr"/>
+      <c r="F1792" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCOCCN(C)C)cc(O)c6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1792" t="inlineStr"/>
+      <c r="H1792" t="inlineStr"/>
+      <c r="I1792" t="n">
+        <v>0.8925505129153195</v>
+      </c>
+      <c r="J1792" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1792" t="inlineStr"/>
+    </row>
+    <row r="1793">
+      <c r="A1793" s="1" t="n">
+        <v>1791</v>
+      </c>
+      <c r="B1793" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0170.png</t>
+        </is>
+      </c>
+      <c r="C1793" t="inlineStr"/>
+      <c r="D1793" t="inlineStr"/>
+      <c r="E1793" t="inlineStr"/>
+      <c r="F1793" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCC7CCCN(C)C7)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1793" t="inlineStr"/>
+      <c r="H1793" t="inlineStr"/>
+      <c r="I1793" t="n">
+        <v>0.9028196903080433</v>
+      </c>
+      <c r="J1793" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1793" t="inlineStr"/>
+    </row>
+    <row r="1794">
+      <c r="A1794" s="1" t="n">
+        <v>1792</v>
+      </c>
+      <c r="B1794" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0172.png</t>
+        </is>
+      </c>
+      <c r="C1794" t="inlineStr"/>
+      <c r="D1794" t="inlineStr"/>
+      <c r="E1794" t="inlineStr"/>
+      <c r="F1794" t="inlineStr">
+        <is>
+          <t>COc1ccc(CCN(CCOCCNc2cccc3c2C(=O)N(C2CCC(=O)NC2=O)C3=O)Cc2ccc(OCc3ccc(Cl)nc3)c(OC)c2)cc1OC</t>
+        </is>
+      </c>
+      <c r="G1794" t="inlineStr"/>
+      <c r="H1794" t="inlineStr"/>
+      <c r="I1794" t="n">
+        <v>0.9138843826444728</v>
+      </c>
+      <c r="J1794" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1794" t="inlineStr"/>
+    </row>
+    <row r="1795">
+      <c r="A1795" s="1" t="n">
+        <v>1793</v>
+      </c>
+      <c r="B1795" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0173.png</t>
+        </is>
+      </c>
+      <c r="C1795" t="inlineStr"/>
+      <c r="D1795" t="inlineStr"/>
+      <c r="E1795" t="inlineStr"/>
+      <c r="F1795" t="inlineStr">
+        <is>
+          <t>CN(CCOc1cc(C(=O)O)cc2c1nc(Cc1ccc3cc1COCCc1cc(Cl)ccc1COc1cccc-3n1)n2C[C@@H]1CCO1)C(=O)OC(C)(C)C</t>
+        </is>
+      </c>
+      <c r="G1795" t="inlineStr"/>
+      <c r="H1795" t="inlineStr"/>
+      <c r="I1795" t="n">
+        <v>0.8779687317387704</v>
+      </c>
+      <c r="J1795" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1795" t="inlineStr"/>
+    </row>
+    <row r="1796">
+      <c r="A1796" s="1" t="n">
+        <v>1794</v>
+      </c>
+      <c r="B1796" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0174.png</t>
+        </is>
+      </c>
+      <c r="C1796" t="inlineStr"/>
+      <c r="D1796" t="inlineStr"/>
+      <c r="E1796" t="inlineStr"/>
+      <c r="F1796" t="inlineStr">
+        <is>
+          <t>CC(C)c1cnn2c(NCc3ccccc3-c3nccc4cc(N5CCC(CN6CCN(c7cc8c(cc7F)C(=O)N(C7CCC(=O)NC7=O)C8=O)CC6)CC5)ccc34)nc(O[C@@H]3CCCNC3)nc12</t>
+        </is>
+      </c>
+      <c r="G1796" t="inlineStr"/>
+      <c r="H1796" t="inlineStr"/>
+      <c r="I1796" t="n">
+        <v>0.8766044480162879</v>
+      </c>
+      <c r="J1796" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1796" t="inlineStr"/>
+    </row>
+    <row r="1797">
+      <c r="A1797" s="1" t="n">
+        <v>1795</v>
+      </c>
+      <c r="B1797" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0175.png</t>
+        </is>
+      </c>
+      <c r="C1797" t="inlineStr"/>
+      <c r="D1797" t="inlineStr"/>
+      <c r="E1797" t="inlineStr"/>
+      <c r="F1797" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCCN)NC(=O)[C@H](CCCN)NCc2cccnc2Sc2c(Cl)ccc(-c3ccc(C(=O)O)cc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1797" t="inlineStr"/>
+      <c r="H1797" t="inlineStr"/>
+      <c r="I1797" t="n">
+        <v>0.8904165011997766</v>
+      </c>
+      <c r="J1797" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1797" t="inlineStr"/>
+    </row>
+    <row r="1798">
+      <c r="A1798" s="1" t="n">
+        <v>1796</v>
+      </c>
+      <c r="B1798" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0176.png</t>
+        </is>
+      </c>
+      <c r="C1798" t="inlineStr"/>
+      <c r="D1798" t="inlineStr"/>
+      <c r="E1798" t="inlineStr"/>
+      <c r="F1798" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)[C@H]4C[C@@H](C(=O)N[C@@H](C(=O)N5C[C@H](O)C[C@@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)C4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1798" t="inlineStr"/>
+      <c r="H1798" t="inlineStr"/>
+      <c r="I1798" t="n">
+        <v>0.8881256975318474</v>
+      </c>
+      <c r="J1798" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1798" t="inlineStr"/>
+    </row>
+    <row r="1799">
+      <c r="A1799" s="1" t="n">
+        <v>1797</v>
+      </c>
+      <c r="B1799" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0177.png</t>
+        </is>
+      </c>
+      <c r="C1799" t="inlineStr"/>
+      <c r="D1799" t="inlineStr"/>
+      <c r="E1799" t="inlineStr"/>
+      <c r="F1799" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4cnc(C(=O)N[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)C)cn4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1799" t="inlineStr"/>
+      <c r="H1799" t="inlineStr"/>
+      <c r="I1799" t="n">
+        <v>0.8731453405423427</v>
+      </c>
+      <c r="J1799" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1799" t="inlineStr"/>
+    </row>
+    <row r="1800">
+      <c r="A1800" s="1" t="n">
+        <v>1798</v>
+      </c>
+      <c r="B1800" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0181.png</t>
+        </is>
+      </c>
+      <c r="C1800" t="inlineStr"/>
+      <c r="D1800" t="inlineStr"/>
+      <c r="E1800" t="inlineStr"/>
+      <c r="F1800" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN(C)C)cc(SC)c6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1800" t="inlineStr"/>
+      <c r="H1800" t="inlineStr"/>
+      <c r="I1800" t="n">
+        <v>0.8759651474609226</v>
+      </c>
+      <c r="J1800" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1800" t="inlineStr"/>
+    </row>
+    <row r="1801">
+      <c r="A1801" s="1" t="n">
+        <v>1799</v>
+      </c>
+      <c r="B1801" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0183.png</t>
+        </is>
+      </c>
+      <c r="C1801" t="inlineStr"/>
+      <c r="D1801" t="inlineStr"/>
+      <c r="E1801" t="inlineStr"/>
+      <c r="F1801" t="inlineStr">
+        <is>
+          <t>COC(=O)c1cc(NC[C@@H]2CCO2)c(NC(=O)Cc2ccc3cc2COCCc2cc(Cl)ccc2COc2cccc-3n2)c(OCCN(C)C(=O)OC(C)(C)C)c1</t>
+        </is>
+      </c>
+      <c r="G1801" t="inlineStr"/>
+      <c r="H1801" t="inlineStr"/>
+      <c r="I1801" t="n">
+        <v>0.8944119519992774</v>
+      </c>
+      <c r="J1801" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1801" t="inlineStr"/>
+    </row>
+    <row r="1802">
+      <c r="A1802" s="1" t="n">
+        <v>1800</v>
+      </c>
+      <c r="B1802" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0184.png</t>
+        </is>
+      </c>
+      <c r="C1802" t="inlineStr"/>
+      <c r="D1802" t="inlineStr"/>
+      <c r="E1802" t="inlineStr"/>
+      <c r="F1802" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc([C@H](C)NC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)c2csc(N3CCN(c4cc(-c5ccccc5O)nnc4N)CC3)n2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1802" t="inlineStr"/>
+      <c r="H1802" t="inlineStr"/>
+      <c r="I1802" t="n">
+        <v>0.8943015243906124</v>
+      </c>
+      <c r="J1802" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1802" t="inlineStr"/>
+    </row>
+    <row r="1803">
+      <c r="A1803" s="1" t="n">
+        <v>1801</v>
+      </c>
+      <c r="B1803" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0185.png</t>
+        </is>
+      </c>
+      <c r="C1803" t="inlineStr"/>
+      <c r="D1803" t="inlineStr"/>
+      <c r="E1803" t="inlineStr"/>
+      <c r="F1803" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)CN[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1803" t="inlineStr"/>
+      <c r="H1803" t="inlineStr"/>
+      <c r="I1803" t="n">
+        <v>0.8762426746106197</v>
+      </c>
+      <c r="J1803" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1803" t="inlineStr"/>
+    </row>
+    <row r="1804">
+      <c r="A1804" s="1" t="n">
+        <v>1802</v>
+      </c>
+      <c r="B1804" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0186.png</t>
+        </is>
+      </c>
+      <c r="C1804" t="inlineStr"/>
+      <c r="D1804" t="inlineStr"/>
+      <c r="E1804" t="inlineStr"/>
+      <c r="F1804" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCOCCN(C)C)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1804" t="inlineStr"/>
+      <c r="H1804" t="inlineStr"/>
+      <c r="I1804" t="n">
+        <v>0.8926495640948178</v>
+      </c>
+      <c r="J1804" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1804" t="inlineStr"/>
+    </row>
+    <row r="1805">
+      <c r="A1805" s="1" t="n">
+        <v>1803</v>
+      </c>
+      <c r="B1805" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0187.png</t>
+        </is>
+      </c>
+      <c r="C1805" t="inlineStr"/>
+      <c r="D1805" t="inlineStr"/>
+      <c r="E1805" t="inlineStr"/>
+      <c r="F1805" t="inlineStr">
+        <is>
+          <t>Cc1cc(-c2ncnc3[nH]c(-c4ccc(C5CCN(CCCC6CN(c7ccc8c(c7)C(=O)N(C7CCC(=O)NC7=O)C8=O)C6)CC5)cc4)cc23)ccc1CNC(=O)c1nc(C(C)(C)C)no1</t>
+        </is>
+      </c>
+      <c r="G1805" t="inlineStr"/>
+      <c r="H1805" t="inlineStr"/>
+      <c r="I1805" t="n">
+        <v>0.8475143245797137</v>
+      </c>
+      <c r="J1805" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1805" t="inlineStr"/>
+    </row>
+    <row r="1806">
+      <c r="A1806" s="1" t="n">
+        <v>1804</v>
+      </c>
+      <c r="B1806" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0189.png</t>
+        </is>
+      </c>
+      <c r="C1806" t="inlineStr"/>
+      <c r="D1806" t="inlineStr"/>
+      <c r="E1806" t="inlineStr"/>
+      <c r="F1806" t="inlineStr">
+        <is>
+          <t>NC(=O)c1c(-c2ccc(Oc3ccccc3)cc2)nn2c1Nc1ccc(C(=O)NC3CCN(CC4CCN(c5cc6c(cc5F)C(=O)N(C5CCC(=O)NC5=O)C6=O)CC4)CC3)cc1CC2</t>
+        </is>
+      </c>
+      <c r="G1806" t="inlineStr"/>
+      <c r="H1806" t="inlineStr"/>
+      <c r="I1806" t="n">
+        <v>0.8915134122491665</v>
+      </c>
+      <c r="J1806" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1806" t="inlineStr"/>
+    </row>
+    <row r="1807">
+      <c r="A1807" s="1" t="n">
+        <v>1805</v>
+      </c>
+      <c r="B1807" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0190.png</t>
+        </is>
+      </c>
+      <c r="C1807" t="inlineStr"/>
+      <c r="D1807" t="inlineStr"/>
+      <c r="E1807" t="inlineStr"/>
+      <c r="F1807" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCN)NC(=O)[C@H](CCCN)NCc2cccnc2Sc2c(Cl)ccc(-c3ccc(C(=O)O)cc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1807" t="inlineStr"/>
+      <c r="H1807" t="inlineStr"/>
+      <c r="I1807" t="n">
+        <v>0.8964843053195026</v>
+      </c>
+      <c r="J1807" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1807" t="inlineStr"/>
+    </row>
+    <row r="1808">
+      <c r="A1808" s="1" t="n">
+        <v>1806</v>
+      </c>
+      <c r="B1808" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0191.png</t>
+        </is>
+      </c>
+      <c r="C1808" t="inlineStr"/>
+      <c r="D1808" t="inlineStr"/>
+      <c r="E1808" t="inlineStr"/>
+      <c r="F1808" t="inlineStr">
+        <is>
+          <t>Cc1cnc(Nc2cc(C3CCN(C(=O)c4cnc(C(=O)Nc5cccc6c5C(=O)N(C5CCC(=O)NC5=O)C6=O)cn4)CC3)cc(N3CCC(F)(F)C3)n2)cn1</t>
+        </is>
+      </c>
+      <c r="G1808" t="inlineStr"/>
+      <c r="H1808" t="inlineStr"/>
+      <c r="I1808" t="n">
+        <v>0.8970650205306012</v>
+      </c>
+      <c r="J1808" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1808" t="inlineStr"/>
+    </row>
+    <row r="1809">
+      <c r="A1809" s="1" t="n">
+        <v>1807</v>
+      </c>
+      <c r="B1809" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0192.png</t>
+        </is>
+      </c>
+      <c r="C1809" t="inlineStr"/>
+      <c r="D1809" t="inlineStr"/>
+      <c r="E1809" t="inlineStr"/>
+      <c r="F1809" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)[C@@H]4CC[C@@H]4C(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1809" t="inlineStr"/>
+      <c r="H1809" t="inlineStr"/>
+      <c r="I1809" t="n">
+        <v>0.8901290210565896</v>
+      </c>
+      <c r="J1809" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1809" t="inlineStr"/>
+    </row>
+    <row r="1810">
+      <c r="A1810" s="1" t="n">
+        <v>1808</v>
+      </c>
+      <c r="B1810" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0196.png</t>
+        </is>
+      </c>
+      <c r="C1810" t="inlineStr"/>
+      <c r="D1810" t="inlineStr"/>
+      <c r="E1810" t="inlineStr"/>
+      <c r="F1810" t="inlineStr">
+        <is>
+          <t>NC(=O)CN1CCN(CC(N)=O)CCN(CC(=O)NCC2CCC(C(=O)NC(Cc3ccc4ccccc4c3)C(=O)NCCCCC(NC(=O)NC(CCC(=O)O)C(=O)O)C(=O)O)CC2)CCN(CC(N)=O)CC1</t>
+        </is>
+      </c>
+      <c r="G1810" t="inlineStr"/>
+      <c r="H1810" t="inlineStr"/>
+      <c r="I1810" t="n">
+        <v>0.8865682031703374</v>
+      </c>
+      <c r="J1810" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1810" t="inlineStr"/>
+    </row>
+    <row r="1811">
+      <c r="A1811" s="1" t="n">
+        <v>1809</v>
+      </c>
+      <c r="B1811" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0197.png</t>
+        </is>
+      </c>
+      <c r="C1811" t="inlineStr"/>
+      <c r="D1811" t="inlineStr"/>
+      <c r="E1811" t="inlineStr"/>
+      <c r="F1811" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(O)cc(F)c6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1811" t="inlineStr"/>
+      <c r="H1811" t="inlineStr"/>
+      <c r="I1811" t="n">
+        <v>0.8936711567255069</v>
+      </c>
+      <c r="J1811" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1811" t="inlineStr"/>
+    </row>
+    <row r="1812">
+      <c r="A1812" s="1" t="n">
+        <v>1810</v>
+      </c>
+      <c r="B1812" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0199.png</t>
+        </is>
+      </c>
+      <c r="C1812" t="inlineStr"/>
+      <c r="D1812" t="inlineStr"/>
+      <c r="E1812" t="inlineStr"/>
+      <c r="F1812" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4ccc(CN[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)cc4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1812" t="inlineStr"/>
+      <c r="H1812" t="inlineStr"/>
+      <c r="I1812" t="n">
+        <v>0.9021786926100969</v>
+      </c>
+      <c r="J1812" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1812" t="inlineStr"/>
+    </row>
+    <row r="1813">
+      <c r="A1813" s="1" t="n">
+        <v>1811</v>
+      </c>
+      <c r="B1813" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0200.png</t>
+        </is>
+      </c>
+      <c r="C1813" t="inlineStr"/>
+      <c r="D1813" t="inlineStr"/>
+      <c r="E1813" t="inlineStr"/>
+      <c r="F1813" t="inlineStr">
+        <is>
+          <t>NC(=O)c1c(-c2ccc(Oc3ccccc3)cc2)nn2c1Nc1ccc(C(=O)N[C@@H]3CC[C@@H](CN4CCN(c5cc6c(cc5F)C(=O)N(C5CCC(=O)NC5=O)C6=O)CC4)CC3)cc1CC2</t>
+        </is>
+      </c>
+      <c r="G1813" t="inlineStr"/>
+      <c r="H1813" t="inlineStr"/>
+      <c r="I1813" t="n">
+        <v>0.8939187520780157</v>
+      </c>
+      <c r="J1813" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1813" t="inlineStr"/>
+    </row>
+    <row r="1814">
+      <c r="A1814" s="1" t="n">
+        <v>1812</v>
+      </c>
+      <c r="B1814" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0201.png</t>
+        </is>
+      </c>
+      <c r="C1814" t="inlineStr"/>
+      <c r="D1814" t="inlineStr"/>
+      <c r="E1814" t="inlineStr"/>
+      <c r="F1814" t="inlineStr">
+        <is>
+          <t>CN1CC[C@H]2CC[C@@H](C(=O)N[C@@H](CCC(N)=O)C(=O)NC(CCC(=O)N3CCC(C#Cc4cccc5c4CN(C4CCC(=O)NC4=O)C5=O)CC3)c3ccccc3)N2C(=O)[C@@H](NC(=O)c2cc3cc(C(F)(F)P(=O)(O)O)ccc3s2)C1</t>
+        </is>
+      </c>
+      <c r="G1814" t="inlineStr"/>
+      <c r="H1814" t="inlineStr"/>
+      <c r="I1814" t="n">
+        <v>0.845426429024724</v>
+      </c>
+      <c r="J1814" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1814" t="inlineStr"/>
+    </row>
+    <row r="1815">
+      <c r="A1815" s="1" t="n">
+        <v>1813</v>
+      </c>
+      <c r="B1815" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0203.png</t>
+        </is>
+      </c>
+      <c r="C1815" t="inlineStr"/>
+      <c r="D1815" t="inlineStr"/>
+      <c r="E1815" t="inlineStr"/>
+      <c r="F1815" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCNC(=O)OC(C)(C)C)NC(=O)[C@H](CCCNC(=O)OC(C)(C)C)NCc2cccnc2Sc2c(Cl)ccc(Br)c2CNC(=O)[C@@H]1Cc1cn(C(=O)OC(C)(C)C)c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1815" t="inlineStr"/>
+      <c r="H1815" t="inlineStr"/>
+      <c r="I1815" t="n">
+        <v>0.8953788666047585</v>
+      </c>
+      <c r="J1815" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1815" t="inlineStr"/>
+    </row>
+    <row r="1816">
+      <c r="A1816" s="1" t="n">
+        <v>1814</v>
+      </c>
+      <c r="B1816" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0205.png</t>
+        </is>
+      </c>
+      <c r="C1816" t="inlineStr"/>
+      <c r="D1816" t="inlineStr"/>
+      <c r="E1816" t="inlineStr"/>
+      <c r="F1816" t="inlineStr">
+        <is>
+          <t>NC(=O)c1c(-c2ccc(Oc3ccccc3)cc2)nn2c1Nc1ccc(C(=O)N3CCN(CC4CCN(c5ccc6c(c5)C(=O)N(C5CCC(=O)NC5=O)C6=O)CC4)CC3)cc1CC2</t>
+        </is>
+      </c>
+      <c r="G1816" t="inlineStr"/>
+      <c r="H1816" t="inlineStr"/>
+      <c r="I1816" t="n">
+        <v>0.8770286103694482</v>
+      </c>
+      <c r="J1816" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1816" t="inlineStr"/>
+    </row>
+    <row r="1817">
+      <c r="A1817" s="1" t="n">
+        <v>1815</v>
+      </c>
+      <c r="B1817" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0206.png</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr"/>
+      <c r="D1817" t="inlineStr"/>
+      <c r="E1817" t="inlineStr"/>
+      <c r="F1817" t="inlineStr">
+        <is>
+          <t>Cc1[nH]c2ccccc2c1C[C@H]1C(=O)NCc2c(-c3ccc(C(=O)O)cc3)ccc(Cl)c2Sc2ncccc2CN[C@@H](CCCN)C(=O)N[C@@H](CCCCN)C(=O)N1C</t>
+        </is>
+      </c>
+      <c r="G1817" t="inlineStr"/>
+      <c r="H1817" t="inlineStr"/>
+      <c r="I1817" t="n">
+        <v>0.9082435204872276</v>
+      </c>
+      <c r="J1817" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1817" t="inlineStr"/>
+    </row>
+    <row r="1818">
+      <c r="A1818" s="1" t="n">
+        <v>1816</v>
+      </c>
+      <c r="B1818" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0207.png</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr"/>
+      <c r="D1818" t="inlineStr"/>
+      <c r="E1818" t="inlineStr"/>
+      <c r="F1818" t="inlineStr">
+        <is>
+          <t>COc1cc(-c2ccc3c(c2)CCCOc2cc(ccc2Cc2nc4ccc(C(=O)O)cc4n2C[C@@H]2CCO2)-c2cccc(n2)OC3)ccn1</t>
+        </is>
+      </c>
+      <c r="G1818" t="inlineStr"/>
+      <c r="H1818" t="inlineStr"/>
+      <c r="I1818" t="n">
+        <v>0.8825812792317952</v>
+      </c>
+      <c r="J1818" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1818" t="inlineStr"/>
+    </row>
+    <row r="1819">
+      <c r="A1819" s="1" t="n">
+        <v>1817</v>
+      </c>
+      <c r="B1819" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0208.png</t>
+        </is>
+      </c>
+      <c r="C1819" t="inlineStr"/>
+      <c r="D1819" t="inlineStr"/>
+      <c r="E1819" t="inlineStr"/>
+      <c r="F1819" t="inlineStr">
+        <is>
+          <t>NC(=O)c1c(-c2ccc(Oc3ccccc3)cc2)nn2c1Nc1ccc(C(=O)N3CCC(CN4CCN(c5cc6c(cc5F)C(=O)N(C5CCC(=O)NC5=O)C6=O)CC4)CC3)cc1CC2</t>
+        </is>
+      </c>
+      <c r="G1819" t="inlineStr"/>
+      <c r="H1819" t="inlineStr"/>
+      <c r="I1819" t="n">
+        <v>0.872482261620968</v>
+      </c>
+      <c r="J1819" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1819" t="inlineStr"/>
+    </row>
+    <row r="1820">
+      <c r="A1820" s="1" t="n">
+        <v>1818</v>
+      </c>
+      <c r="B1820" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0209.png</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr"/>
+      <c r="D1820" t="inlineStr"/>
+      <c r="E1820" t="inlineStr"/>
+      <c r="F1820" t="inlineStr">
+        <is>
+          <t>COc1cc(C(=O)NS(=O)(=O)CC2CC2)cc2c1nc(Cc1cc(C)c3cc1OCCCc1cc(F)ccc1COc1cccc-3n1)n2C[C@@H]1CCO1</t>
+        </is>
+      </c>
+      <c r="G1820" t="inlineStr"/>
+      <c r="H1820" t="inlineStr"/>
+      <c r="I1820" t="n">
+        <v>0.8983863462880408</v>
+      </c>
+      <c r="J1820" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1820" t="inlineStr"/>
+    </row>
+    <row r="1821">
+      <c r="A1821" s="1" t="n">
+        <v>1819</v>
+      </c>
+      <c r="B1821" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0211.png</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr"/>
+      <c r="D1821" t="inlineStr"/>
+      <c r="E1821" t="inlineStr"/>
+      <c r="F1821" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN7CCCCC7)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1821" t="inlineStr"/>
+      <c r="H1821" t="inlineStr"/>
+      <c r="I1821" t="n">
+        <v>0.8959538706212233</v>
+      </c>
+      <c r="J1821" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1821" t="inlineStr"/>
+    </row>
+    <row r="1822">
+      <c r="A1822" s="1" t="n">
+        <v>1820</v>
+      </c>
+      <c r="B1822" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0213.png</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr"/>
+      <c r="D1822" t="inlineStr"/>
+      <c r="E1822" t="inlineStr"/>
+      <c r="F1822" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(c3C2=O)C(=O)C=C(NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C)C4=O</t>
+        </is>
+      </c>
+      <c r="G1822" t="inlineStr"/>
+      <c r="H1822" t="inlineStr"/>
+      <c r="I1822" t="n">
+        <v>0.8658190715344175</v>
+      </c>
+      <c r="J1822" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1822" t="inlineStr"/>
+    </row>
+    <row r="1823">
+      <c r="A1823" s="1" t="n">
+        <v>1821</v>
+      </c>
+      <c r="B1823" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0216.png</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr"/>
+      <c r="D1823" t="inlineStr"/>
+      <c r="E1823" t="inlineStr"/>
+      <c r="F1823" t="inlineStr">
+        <is>
+          <t>NC(=O)c1ncc(N2CCCCC2)nc1Nc1ccc(C2CCN(CCCCN(CCC3CCN(C[C@@H]4CC[C@@H](n5cc(NC(=O)c6cnn7ccc(N8CCOCC8)nc67)c(C(F)F)n5)CC4)CC3)c3cccc4c3C(=O)N(C3CCC(=O)NC3=O)C4=O)CC2)cc1</t>
+        </is>
+      </c>
+      <c r="G1823" t="inlineStr"/>
+      <c r="H1823" t="inlineStr"/>
+      <c r="I1823" t="n">
+        <v>0.8993106927911703</v>
+      </c>
+      <c r="J1823" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1823" t="inlineStr"/>
+    </row>
+    <row r="1824">
+      <c r="A1824" s="1" t="n">
+        <v>1822</v>
+      </c>
+      <c r="B1824" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0218.png</t>
+        </is>
+      </c>
+      <c r="C1824" t="inlineStr"/>
+      <c r="D1824" t="inlineStr"/>
+      <c r="E1824" t="inlineStr"/>
+      <c r="F1824" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccc2c(c1)CCCOc1cc(ccc1Cc1nc3c(OCC(=O)N(C)C)cc(C(=O)O)cc3n1C[C@@H]1CCO1)-c1cccc(n1)OC2</t>
+        </is>
+      </c>
+      <c r="G1824" t="inlineStr"/>
+      <c r="H1824" t="inlineStr"/>
+      <c r="I1824" t="n">
+        <v>0.8698908539938425</v>
+      </c>
+      <c r="J1824" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1824" t="inlineStr"/>
+    </row>
+    <row r="1825">
+      <c r="A1825" s="1" t="n">
+        <v>1823</v>
+      </c>
+      <c r="B1825" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0219.png</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr"/>
+      <c r="D1825" t="inlineStr"/>
+      <c r="E1825" t="inlineStr"/>
+      <c r="F1825" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCN)NC(=O)[C@H](CCCN)NCc2cccnc2Sc2c(Cl)ccc(-c3ccc(C(=O)O)cc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1825" t="inlineStr"/>
+      <c r="H1825" t="inlineStr"/>
+      <c r="I1825" t="n">
+        <v>0.8862883111479054</v>
+      </c>
+      <c r="J1825" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1825" t="inlineStr"/>
+    </row>
+    <row r="1826">
+      <c r="A1826" s="1" t="n">
+        <v>1824</v>
+      </c>
+      <c r="B1826" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0221.png</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr"/>
+      <c r="D1826" t="inlineStr"/>
+      <c r="E1826" t="inlineStr"/>
+      <c r="F1826" t="inlineStr">
+        <is>
+          <t>CC(C)c1cnn2c(NCc3ccccc3-c3nccc4cc(NC(=O)/C=C/CN(C)CCOCCOCCOCCNC(=O)CNc5cccc6c5C(=O)N(C5CCC(=O)NC5=O)C6=O)ccc34)nc(N3CCC(N)CC3)nc12</t>
+        </is>
+      </c>
+      <c r="G1826" t="inlineStr"/>
+      <c r="H1826" t="inlineStr"/>
+      <c r="I1826" t="n">
+        <v>0.888811140587797</v>
+      </c>
+      <c r="J1826" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1826" t="inlineStr"/>
+    </row>
+    <row r="1827">
+      <c r="A1827" s="1" t="n">
+        <v>1825</v>
+      </c>
+      <c r="B1827" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0227.png</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr"/>
+      <c r="D1827" t="inlineStr"/>
+      <c r="E1827" t="inlineStr"/>
+      <c r="F1827" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2cc3c(cc2OC)C2(OC3=O)c3cc(-c4ccccc4)c(OC(C)=O)cc3Oc3cc(OC(C)=O)c(-c4ccccc4)cc32)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1827" t="inlineStr"/>
+      <c r="H1827" t="inlineStr"/>
+      <c r="I1827" t="n">
+        <v>0.8860820415074333</v>
+      </c>
+      <c r="J1827" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1827" t="inlineStr"/>
+    </row>
+    <row r="1828">
+      <c r="A1828" s="1" t="n">
+        <v>1826</v>
+      </c>
+      <c r="B1828" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0228.png</t>
+        </is>
+      </c>
+      <c r="C1828" t="inlineStr"/>
+      <c r="D1828" t="inlineStr"/>
+      <c r="E1828" t="inlineStr"/>
+      <c r="F1828" t="inlineStr">
+        <is>
+          <t>COCCOc1cc(C(=O)OC)cc2c1nc(Cc1cc(F)c3cc1CCOCc1cc(ccc1Cl)COc1cccc-3n1)n2C[C@H]1CCO1</t>
+        </is>
+      </c>
+      <c r="G1828" t="inlineStr"/>
+      <c r="H1828" t="inlineStr"/>
+      <c r="I1828" t="n">
+        <v>0.8813598458127065</v>
+      </c>
+      <c r="J1828" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1828" t="inlineStr"/>
+    </row>
+    <row r="1829">
+      <c r="A1829" s="1" t="n">
+        <v>1827</v>
+      </c>
+      <c r="B1829" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0229.png</t>
+        </is>
+      </c>
+      <c r="C1829" t="inlineStr"/>
+      <c r="D1829" t="inlineStr"/>
+      <c r="E1829" t="inlineStr"/>
+      <c r="F1829" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCCNC(=O)OC(C)(C)C)NC(=O)[C@H](CCNC(=O)C(C)(C)C)NCc2cccnc2Sc2c(Cl)ccc(Br)c2CNC(=O)[C@@H]1Cc1cn(C(=O)OC(C)(C)C)c2ccccc12.[HH].[HH]</t>
+        </is>
+      </c>
+      <c r="G1829" t="inlineStr"/>
+      <c r="H1829" t="inlineStr"/>
+      <c r="I1829" t="n">
+        <v>0.8983537709777016</v>
+      </c>
+      <c r="J1829" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1829" t="inlineStr"/>
+    </row>
+    <row r="1830">
+      <c r="A1830" s="1" t="n">
+        <v>1828</v>
+      </c>
+      <c r="B1830" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0232.png</t>
+        </is>
+      </c>
+      <c r="C1830" t="inlineStr"/>
+      <c r="D1830" t="inlineStr"/>
+      <c r="E1830" t="inlineStr"/>
+      <c r="F1830" t="inlineStr">
+        <is>
+          <t>COC(=O)c1cc(OCCO[Si](C)(C)C(C)(C)C)c2nc(Cc3ccc4cc3COCCc3cc(Cl)ccc3COc3cccc-4n3)n(C[C@@H]3CCO3)c2c1</t>
+        </is>
+      </c>
+      <c r="G1830" t="inlineStr"/>
+      <c r="H1830" t="inlineStr"/>
+      <c r="I1830" t="n">
+        <v>0.8976589131581323</v>
+      </c>
+      <c r="J1830" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1830" t="inlineStr"/>
+    </row>
+    <row r="1831">
+      <c r="A1831" s="1" t="n">
+        <v>1829</v>
+      </c>
+      <c r="B1831" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0234.png</t>
+        </is>
+      </c>
+      <c r="C1831" t="inlineStr"/>
+      <c r="D1831" t="inlineStr"/>
+      <c r="E1831" t="inlineStr"/>
+      <c r="F1831" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2cc3c(cc2OC)C2(OC3=O)c3cc(F)c(OC(C)=O)cc3Oc3cc(OC(C)=O)c(F)cc32)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1831" t="inlineStr"/>
+      <c r="H1831" t="inlineStr"/>
+      <c r="I1831" t="n">
+        <v>0.8973909389775973</v>
+      </c>
+      <c r="J1831" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1831" t="inlineStr"/>
+    </row>
+    <row r="1832">
+      <c r="A1832" s="1" t="n">
+        <v>1830</v>
+      </c>
+      <c r="B1832" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0235.png</t>
+        </is>
+      </c>
+      <c r="C1832" t="inlineStr"/>
+      <c r="D1832" t="inlineStr"/>
+      <c r="E1832" t="inlineStr"/>
+      <c r="F1832" t="inlineStr">
+        <is>
+          <t>N#C[C@@H]1CC(F)(F)CN1C(=O)CNC(=O)c1ccnc2c(NC(=O)CCC(=O)NCCNC(=O)CCC(C(=O)O)N3CCN(CC(=O)O)CCN(CC(=O)O)CCN(CC(=O)O)CC3)cccc12</t>
+        </is>
+      </c>
+      <c r="G1832" t="inlineStr"/>
+      <c r="H1832" t="inlineStr"/>
+      <c r="I1832" t="n">
+        <v>0.8740124077418417</v>
+      </c>
+      <c r="J1832" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1832" t="inlineStr"/>
+    </row>
+    <row r="1833">
+      <c r="A1833" s="1" t="n">
+        <v>1831</v>
+      </c>
+      <c r="B1833" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0238.png</t>
+        </is>
+      </c>
+      <c r="C1833" t="inlineStr"/>
+      <c r="D1833" t="inlineStr"/>
+      <c r="E1833" t="inlineStr"/>
+      <c r="F1833" t="inlineStr">
+        <is>
+          <t>Cc1ccc(S(=O)(=O)Nc2ccc(C[C@H](N)C(=O)N3CCC(CCC#Cc4cccc5c4CN(C4CCC(=O)NC4=O)C5=O)CC3)cc2)cc1</t>
+        </is>
+      </c>
+      <c r="G1833" t="inlineStr"/>
+      <c r="H1833" t="inlineStr"/>
+      <c r="I1833" t="n">
+        <v>0.8923162527711789</v>
+      </c>
+      <c r="J1833" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1833" t="inlineStr"/>
+    </row>
+    <row r="1834">
+      <c r="A1834" s="1" t="n">
+        <v>1832</v>
+      </c>
+      <c r="B1834" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0239.png</t>
+        </is>
+      </c>
+      <c r="C1834" t="inlineStr"/>
+      <c r="D1834" t="inlineStr"/>
+      <c r="E1834" t="inlineStr"/>
+      <c r="F1834" t="inlineStr">
+        <is>
+          <t>Cc1[nH]c2ccccc2c1C[C@H]1C(=O)NCc2c(cccc2-c2ccc(C(=O)O)cc2)Sc2ncccc2CN[C@@H](CCCN)C(=O)N[C@@H](CCCCN)C(=O)N1C</t>
+        </is>
+      </c>
+      <c r="G1834" t="inlineStr"/>
+      <c r="H1834" t="inlineStr"/>
+      <c r="I1834" t="n">
+        <v>0.9116286421505283</v>
+      </c>
+      <c r="J1834" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1834" t="inlineStr"/>
+    </row>
+    <row r="1835">
+      <c r="A1835" s="1" t="n">
+        <v>1833</v>
+      </c>
+      <c r="B1835" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0240.png</t>
+        </is>
+      </c>
+      <c r="C1835" t="inlineStr"/>
+      <c r="D1835" t="inlineStr"/>
+      <c r="E1835" t="inlineStr"/>
+      <c r="F1835" t="inlineStr">
+        <is>
+          <t>CN1CCC(CNC(=O)c2ccc(C[C@H](N)C(=O)N3CCC(CCC#Cc4cccc5c4CN(C4CCC(=O)NC4=O)C5=O)CC3)cc2)CC1</t>
+        </is>
+      </c>
+      <c r="G1835" t="inlineStr"/>
+      <c r="H1835" t="inlineStr"/>
+      <c r="I1835" t="n">
+        <v>0.8821742390197592</v>
+      </c>
+      <c r="J1835" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1835" t="inlineStr"/>
+    </row>
+    <row r="1836">
+      <c r="A1836" s="1" t="n">
+        <v>1834</v>
+      </c>
+      <c r="B1836" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0241.png</t>
+        </is>
+      </c>
+      <c r="C1836" t="inlineStr"/>
+      <c r="D1836" t="inlineStr"/>
+      <c r="E1836" t="inlineStr"/>
+      <c r="F1836" t="inlineStr">
+        <is>
+          <t>COCCOc1cc(C(=O)OC)cc2c1nc(Cc1ccc3cc1COCCc1cc(ccc1C#N)COc1cccc-3n1)n2C[C@@H]1CCO1</t>
+        </is>
+      </c>
+      <c r="G1836" t="inlineStr"/>
+      <c r="H1836" t="inlineStr"/>
+      <c r="I1836" t="n">
+        <v>0.895511138065637</v>
+      </c>
+      <c r="J1836" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1836" t="inlineStr"/>
+    </row>
+    <row r="1837">
+      <c r="A1837" s="1" t="n">
+        <v>1835</v>
+      </c>
+      <c r="B1837" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0242.png</t>
+        </is>
+      </c>
+      <c r="C1837" t="inlineStr"/>
+      <c r="D1837" t="inlineStr"/>
+      <c r="E1837" t="inlineStr"/>
+      <c r="F1837" t="inlineStr">
+        <is>
+          <t>COCCOc1cc(C(=O)OC)cc2c1nc(Cc1ccc3cc1COCCc1nc(ccc1C#N)COc1cccc-3n1)n2C[C@@H]1CCO1</t>
+        </is>
+      </c>
+      <c r="G1837" t="inlineStr"/>
+      <c r="H1837" t="inlineStr"/>
+      <c r="I1837" t="n">
+        <v>0.8627408265652562</v>
+      </c>
+      <c r="J1837" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1837" t="inlineStr"/>
+    </row>
+    <row r="1838">
+      <c r="A1838" s="1" t="n">
+        <v>1836</v>
+      </c>
+      <c r="B1838" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0243.png</t>
+        </is>
+      </c>
+      <c r="C1838" t="inlineStr"/>
+      <c r="D1838" t="inlineStr"/>
+      <c r="E1838" t="inlineStr"/>
+      <c r="F1838" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN(C)C)cc(S(C)(=O)=O)c6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1838" t="inlineStr"/>
+      <c r="H1838" t="inlineStr"/>
+      <c r="I1838" t="n">
+        <v>0.8732411923641403</v>
+      </c>
+      <c r="J1838" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1838" t="inlineStr"/>
+    </row>
+    <row r="1839">
+      <c r="A1839" s="1" t="n">
+        <v>1837</v>
+      </c>
+      <c r="B1839" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0245.png</t>
+        </is>
+      </c>
+      <c r="C1839" t="inlineStr"/>
+      <c r="D1839" t="inlineStr"/>
+      <c r="E1839" t="inlineStr"/>
+      <c r="F1839" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCn7ccnc7)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1839" t="inlineStr"/>
+      <c r="H1839" t="inlineStr"/>
+      <c r="I1839" t="n">
+        <v>0.8955935207794978</v>
+      </c>
+      <c r="J1839" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1839" t="inlineStr"/>
+    </row>
+    <row r="1840">
+      <c r="A1840" s="1" t="n">
+        <v>1838</v>
+      </c>
+      <c r="B1840" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0246.png</t>
+        </is>
+      </c>
+      <c r="C1840" t="inlineStr"/>
+      <c r="D1840" t="inlineStr"/>
+      <c r="E1840" t="inlineStr"/>
+      <c r="F1840" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCCN)NC(=O)[C@H](CCC(N)=O)NCc2cccnc2Sc2c(Cl)ccc(-c3ccc(C(=O)O)cc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1840" t="inlineStr"/>
+      <c r="H1840" t="inlineStr"/>
+      <c r="I1840" t="n">
+        <v>0.9060925574269924</v>
+      </c>
+      <c r="J1840" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1840" t="inlineStr"/>
+    </row>
+    <row r="1841">
+      <c r="A1841" s="1" t="n">
+        <v>1839</v>
+      </c>
+      <c r="B1841" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0247.png</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr"/>
+      <c r="D1841" t="inlineStr"/>
+      <c r="E1841" t="inlineStr"/>
+      <c r="F1841" t="inlineStr">
+        <is>
+          <t>C[CH][C@H](O)[C@H](C)[C@@H](O)[C@@H](C)/C=C/C=C(/C)C(=O)Nc1c2oc3cc(OCCNC(C)=O)ccc3nc-2c2c3c(c(C)c(O)c2c1=O)O[C@](C)(O/C=C/[CH]OC)C3=O |^1:1,52|</t>
+        </is>
+      </c>
+      <c r="G1841" t="inlineStr"/>
+      <c r="H1841" t="inlineStr"/>
+      <c r="I1841" t="n">
+        <v>0.8871420559330476</v>
+      </c>
+      <c r="J1841" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1841" t="inlineStr"/>
+    </row>
+    <row r="1842">
+      <c r="A1842" s="1" t="n">
+        <v>1840</v>
+      </c>
+      <c r="B1842" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0250.png</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr"/>
+      <c r="D1842" t="inlineStr"/>
+      <c r="E1842" t="inlineStr"/>
+      <c r="F1842" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2cc3c(cc2OC)C2(OC3=O)c3cc(OC)c(OC(C)=O)c(Cl)c3Oc3c2cc(OC)c(OC(C)=O)c3Cl)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1842" t="inlineStr"/>
+      <c r="H1842" t="inlineStr"/>
+      <c r="I1842" t="n">
+        <v>0.8620903665103316</v>
+      </c>
+      <c r="J1842" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1842" t="inlineStr"/>
+    </row>
+    <row r="1843">
+      <c r="A1843" s="1" t="n">
+        <v>1841</v>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0252.png</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr"/>
+      <c r="D1843" t="inlineStr"/>
+      <c r="E1843" t="inlineStr"/>
+      <c r="F1843" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5n(C)c6cc(O)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1843" t="inlineStr"/>
+      <c r="H1843" t="inlineStr"/>
+      <c r="I1843" t="n">
+        <v>0.8687157644785235</v>
+      </c>
+      <c r="J1843" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1843" t="inlineStr"/>
+    </row>
+    <row r="1844">
+      <c r="A1844" s="1" t="n">
+        <v>1842</v>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0254.png</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr"/>
+      <c r="D1844" t="inlineStr"/>
+      <c r="E1844" t="inlineStr"/>
+      <c r="F1844" t="inlineStr">
+        <is>
+          <t>O=C(O)c1ccc2nc(Cc3ccc4cc3OCCCc3cc(-c5cnn(C6COC6)c5)ccc3COc3cccc-4n3)n(C[C@@H]3CCO3)c2c1</t>
+        </is>
+      </c>
+      <c r="G1844" t="inlineStr"/>
+      <c r="H1844" t="inlineStr"/>
+      <c r="I1844" t="n">
+        <v>0.8904506807236929</v>
+      </c>
+      <c r="J1844" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1844" t="inlineStr"/>
+    </row>
+    <row r="1845">
+      <c r="A1845" s="1" t="n">
+        <v>1843</v>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0255.png</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr"/>
+      <c r="D1845" t="inlineStr"/>
+      <c r="E1845" t="inlineStr"/>
+      <c r="F1845" t="inlineStr">
+        <is>
+          <t>CC(C)c1cnn2c(NCc3ccccc3-c3nccc4cc(NC(=O)/C=C/CN(C)CCOCCNC(=O)CNc5cccc6c5C(=O)N(C5CCC(=O)NC5=O)C6=O)ccc34)nc(N3CCC(N)CC3)nc12</t>
+        </is>
+      </c>
+      <c r="G1845" t="inlineStr"/>
+      <c r="H1845" t="inlineStr"/>
+      <c r="I1845" t="n">
+        <v>0.892078137247225</v>
+      </c>
+      <c r="J1845" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1845" t="inlineStr"/>
+    </row>
+    <row r="1846">
+      <c r="A1846" s="1" t="n">
+        <v>1844</v>
+      </c>
+      <c r="B1846" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0256.png</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr"/>
+      <c r="D1846" t="inlineStr"/>
+      <c r="E1846" t="inlineStr"/>
+      <c r="F1846" t="inlineStr">
+        <is>
+          <t>CC(C)(O)c1cc2nn(C3CCC(CN4CC5(CC(C(CNc6cccc7c6C(=O)N(C6CCC(=O)NC6=O)C7=O)CN6CCC(c7ccc(Nc8nc(N9CCCCC9)cnc8C(N)=O)cc7)CC6)C5)C4)CC3)cc2cc1NC(=O)c1cccc(C(F)(F)F)n1</t>
+        </is>
+      </c>
+      <c r="G1846" t="inlineStr"/>
+      <c r="H1846" t="inlineStr"/>
+      <c r="I1846" t="n">
+        <v>0.8763772623109352</v>
+      </c>
+      <c r="J1846" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1846" t="inlineStr"/>
+    </row>
+    <row r="1847">
+      <c r="A1847" s="1" t="n">
+        <v>1845</v>
+      </c>
+      <c r="B1847" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0259.png</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr"/>
+      <c r="D1847" t="inlineStr"/>
+      <c r="E1847" t="inlineStr"/>
+      <c r="F1847" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCNC(=O)OC(C)(C)C)NC(=O)[C@H](CCNC(=O)C(C)(C)C)NCc2cccnc2Sc2c(Cl)ccc(Br)c2CNC(=O)[C@@H]1Cc1cn(C(=O)OC(C)(C)C)c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1847" t="inlineStr"/>
+      <c r="H1847" t="inlineStr"/>
+      <c r="I1847" t="n">
+        <v>0.9010334931058321</v>
+      </c>
+      <c r="J1847" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1847" t="inlineStr"/>
+    </row>
+    <row r="1848">
+      <c r="A1848" s="1" t="n">
+        <v>1846</v>
+      </c>
+      <c r="B1848" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0260.png</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr"/>
+      <c r="D1848" t="inlineStr"/>
+      <c r="E1848" t="inlineStr"/>
+      <c r="F1848" t="inlineStr">
+        <is>
+          <t>CN[C@@H](C)C(=O)N[C@H]1CN(S(=O)(=O)c2cccc(S(=O)(=O)N3CC[C@H]4CC[C@@H](C(=O)NC(c5ccccc5)c5ccccc5)N4C(=O)[C@@H](NC(=O)[C@H](C)NC)C3)c2)CC[C@H]2CC[C@@H](C(=O)NC(c3ccccc3)c3ccccc3)N2C1=O</t>
+        </is>
+      </c>
+      <c r="G1848" t="inlineStr"/>
+      <c r="H1848" t="inlineStr"/>
+      <c r="I1848" t="n">
+        <v>0.8686951276643128</v>
+      </c>
+      <c r="J1848" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1848" t="inlineStr"/>
+    </row>
+    <row r="1849">
+      <c r="A1849" s="1" t="n">
+        <v>1847</v>
+      </c>
+      <c r="B1849" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0262.png</t>
+        </is>
+      </c>
+      <c r="C1849" t="inlineStr"/>
+      <c r="D1849" t="inlineStr"/>
+      <c r="E1849" t="inlineStr"/>
+      <c r="F1849" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc([C@H](C)NC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)CCCCCCC(=O)N2CCC(c3cc(Nc4cnccn4)nc(N4CCC(F)(F)C4)c3)CC2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1849" t="inlineStr"/>
+      <c r="H1849" t="inlineStr"/>
+      <c r="I1849" t="n">
+        <v>0.887019591997399</v>
+      </c>
+      <c r="J1849" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1849" t="inlineStr"/>
+    </row>
+    <row r="1850">
+      <c r="A1850" s="1" t="n">
+        <v>1848</v>
+      </c>
+      <c r="B1850" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0263.png</t>
+        </is>
+      </c>
+      <c r="C1850" t="inlineStr"/>
+      <c r="D1850" t="inlineStr"/>
+      <c r="E1850" t="inlineStr"/>
+      <c r="F1850" t="inlineStr">
+        <is>
+          <t>COc1ccc(-c2ccc(C(=O)O)cc2)c2c1Sc1ncccc1CN[C@@H](CCCN)C(=O)N[C@@H](CCCCN)C(=O)N(C)[C@@H](Cc1c[nH]c3ccccc13)C(=O)NC2</t>
+        </is>
+      </c>
+      <c r="G1850" t="inlineStr"/>
+      <c r="H1850" t="inlineStr"/>
+      <c r="I1850" t="n">
+        <v>0.8653530536302241</v>
+      </c>
+      <c r="J1850" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1850" t="inlineStr"/>
+    </row>
+    <row r="1851">
+      <c r="A1851" s="1" t="n">
+        <v>1849</v>
+      </c>
+      <c r="B1851" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0264.png</t>
+        </is>
+      </c>
+      <c r="C1851" t="inlineStr"/>
+      <c r="D1851" t="inlineStr"/>
+      <c r="E1851" t="inlineStr"/>
+      <c r="F1851" t="inlineStr">
+        <is>
+          <t>Cc1cnc(Nc2cc(C3CCN(C(=O)COc4cccc5c4C(=O)N(C4CCC(=O)NC4=O)C5=O)CC3)cc(N3CCC(F)(F)C3)n2)cn1</t>
+        </is>
+      </c>
+      <c r="G1851" t="inlineStr"/>
+      <c r="H1851" t="inlineStr"/>
+      <c r="I1851" t="n">
+        <v>0.8901492951147394</v>
+      </c>
+      <c r="J1851" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1851" t="inlineStr"/>
+    </row>
+    <row r="1852">
+      <c r="A1852" s="1" t="n">
+        <v>1850</v>
+      </c>
+      <c r="B1852" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0268.png</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr"/>
+      <c r="D1852" t="inlineStr"/>
+      <c r="E1852" t="inlineStr"/>
+      <c r="F1852" t="inlineStr">
+        <is>
+          <t>CO[C@H]1C[C@@H]2CC[C@@H](C)[C@@](O)(O2)C(=O)C(=O)N2CCCC[C@H]2C(=O)O[C@H]([C@H](C)C[C@@H]2CC[C@H](n3cnnn3)[C@H](OC)C2)CC(=O)[C@H](C)/C=C(\C)[C@@H](O)[C@@H](OC)C(=O)[C@H](C)C[C@H](C)/C=C/C=C/C=C/1C</t>
+        </is>
+      </c>
+      <c r="G1852" t="inlineStr"/>
+      <c r="H1852" t="inlineStr"/>
+      <c r="I1852" t="n">
+        <v>0.8823610976819186</v>
+      </c>
+      <c r="J1852" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1852" t="inlineStr"/>
+    </row>
+    <row r="1853">
+      <c r="A1853" s="1" t="n">
+        <v>1851</v>
+      </c>
+      <c r="B1853" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0269.png</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr"/>
+      <c r="D1853" t="inlineStr"/>
+      <c r="E1853" t="inlineStr"/>
+      <c r="F1853" t="inlineStr">
+        <is>
+          <t>NC(=O)c1c(-c2ccc(Oc3ccccc3)cc2)nn2c1Nc1ccc(NC(=O)C3CCN(c4ccc5c(c4)C(=O)N(C4CCC(=O)NC4=O)C5=O)CC3)cc1CC2</t>
+        </is>
+      </c>
+      <c r="G1853" t="inlineStr"/>
+      <c r="H1853" t="inlineStr"/>
+      <c r="I1853" t="n">
+        <v>0.8922588532817833</v>
+      </c>
+      <c r="J1853" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1853" t="inlineStr"/>
+    </row>
+    <row r="1854">
+      <c r="A1854" s="1" t="n">
+        <v>1852</v>
+      </c>
+      <c r="B1854" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0270.png</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr"/>
+      <c r="D1854" t="inlineStr"/>
+      <c r="E1854" t="inlineStr"/>
+      <c r="F1854" t="inlineStr">
+        <is>
+          <t>CC(C)c1cnn2c(NCc3ccccc3-c3nccc4c3C=CC(N3CCN(CC5CCN(c6ccc7c(c6)C(=O)N(C6CCC(=O)NC6=O)C7=O)CC5)CC3)C4)nc(O[C@@H]3CCCNC3)nc12</t>
+        </is>
+      </c>
+      <c r="G1854" t="inlineStr"/>
+      <c r="H1854" t="inlineStr"/>
+      <c r="I1854" t="n">
+        <v>0.9028264859906784</v>
+      </c>
+      <c r="J1854" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1854" t="inlineStr"/>
+    </row>
+    <row r="1855">
+      <c r="A1855" s="1" t="n">
+        <v>1853</v>
+      </c>
+      <c r="B1855" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0271.png</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr"/>
+      <c r="D1855" t="inlineStr"/>
+      <c r="E1855" t="inlineStr"/>
+      <c r="F1855" t="inlineStr">
+        <is>
+          <t>Cn1cc(-c2ccc3c(c2)CCCOc2cc(ccc2Cc2nc4ccc(C(=O)O)cc4n2C[C@@H]2CCO2)-c2cccc(n2)OC3)ccc1=O</t>
+        </is>
+      </c>
+      <c r="G1855" t="inlineStr"/>
+      <c r="H1855" t="inlineStr"/>
+      <c r="I1855" t="n">
+        <v>0.8748284702461027</v>
+      </c>
+      <c r="J1855" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1855" t="inlineStr"/>
+    </row>
+    <row r="1856">
+      <c r="A1856" s="1" t="n">
+        <v>1854</v>
+      </c>
+      <c r="B1856" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0272.png</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr"/>
+      <c r="D1856" t="inlineStr"/>
+      <c r="E1856" t="inlineStr"/>
+      <c r="F1856" t="inlineStr">
+        <is>
+          <t>COCCOc1cc(C(=O)OC)cc2c1nc(Cc1cc(F)c3cc1COCCc1cc(ccc1C#N)COc1cccc-3n1)n2C[C@@H]1CCO1</t>
+        </is>
+      </c>
+      <c r="G1856" t="inlineStr"/>
+      <c r="H1856" t="inlineStr"/>
+      <c r="I1856" t="n">
+        <v>0.9039156002199558</v>
+      </c>
+      <c r="J1856" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1856" t="inlineStr"/>
+    </row>
+    <row r="1857">
+      <c r="A1857" s="1" t="n">
+        <v>1855</v>
+      </c>
+      <c r="B1857" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0274.png</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr"/>
+      <c r="D1857" t="inlineStr"/>
+      <c r="E1857" t="inlineStr"/>
+      <c r="F1857" t="inlineStr">
+        <is>
+          <t>O=C(O)COC1=CC(C2=C3C=CC(C=CC4=CC=CC=C4)=N3Br(F)(F)N3C(C=CC4=CC=CC=C4)=CC=C23)=CC=C1N1CCOCCOCCN(C2=C(OCC(=O)O)C=CC=C2)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1857" t="inlineStr"/>
+      <c r="H1857" t="inlineStr"/>
+      <c r="I1857" t="n">
+        <v>0.8881617555437529</v>
+      </c>
+      <c r="J1857" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1857" t="inlineStr"/>
+    </row>
+    <row r="1858">
+      <c r="A1858" s="1" t="n">
+        <v>1856</v>
+      </c>
+      <c r="B1858" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0277.png</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr"/>
+      <c r="D1858" t="inlineStr"/>
+      <c r="E1858" t="inlineStr"/>
+      <c r="F1858" t="inlineStr">
+        <is>
+          <t>CC(C)(O)c1cc2nc([C@@H]3CC[C@@H](CN4CCC(CCN(CCCCN5CCC(c6ccc(Nc7nc(N8CCCCC8)cnc7C(N)=O)cc6)CC5)c5cccc6c5C(=O)N(C5CCC(=O)NC5=O)C6=O)CC4)CC3)sc2cc1NC(=O)c1cccc(C(F)(F)F)n1</t>
+        </is>
+      </c>
+      <c r="G1858" t="inlineStr"/>
+      <c r="H1858" t="inlineStr"/>
+      <c r="I1858" t="n">
+        <v>0.9032043512469488</v>
+      </c>
+      <c r="J1858" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1858" t="inlineStr"/>
+    </row>
+    <row r="1859">
+      <c r="A1859" s="1" t="n">
+        <v>1857</v>
+      </c>
+      <c r="B1859" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0278.png</t>
+        </is>
+      </c>
+      <c r="C1859" t="inlineStr"/>
+      <c r="D1859" t="inlineStr"/>
+      <c r="E1859" t="inlineStr"/>
+      <c r="F1859" t="inlineStr">
+        <is>
+          <t>O=C(CCOCCOCCOCCOCCC(=O)N1CCC(c2cc(Nc3cc(C(F)(F)F)ccn3)nc(N3CCC(F)(F)C3)c2)CC1)NCCCCNC(=O)CNc1cccc2c1C(=O)N(C1CCC(=O)NC1=O)C2=O</t>
+        </is>
+      </c>
+      <c r="G1859" t="inlineStr"/>
+      <c r="H1859" t="inlineStr"/>
+      <c r="I1859" t="n">
+        <v>0.8569970886044792</v>
+      </c>
+      <c r="J1859" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1859" t="inlineStr"/>
+    </row>
+    <row r="1860">
+      <c r="A1860" s="1" t="n">
+        <v>1858</v>
+      </c>
+      <c r="B1860" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0279.png</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr"/>
+      <c r="D1860" t="inlineStr"/>
+      <c r="E1860" t="inlineStr"/>
+      <c r="F1860" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)[C@H]4CC[C@@H]4C(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1860" t="inlineStr"/>
+      <c r="H1860" t="inlineStr"/>
+      <c r="I1860" t="n">
+        <v>0.8922005901509127</v>
+      </c>
+      <c r="J1860" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1860" t="inlineStr"/>
+    </row>
+    <row r="1861">
+      <c r="A1861" s="1" t="n">
+        <v>1859</v>
+      </c>
+      <c r="B1861" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0281.png</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr"/>
+      <c r="D1861" t="inlineStr"/>
+      <c r="E1861" t="inlineStr"/>
+      <c r="F1861" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4ccc(C(=O)N[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)cc4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1861" t="inlineStr"/>
+      <c r="H1861" t="inlineStr"/>
+      <c r="I1861" t="n">
+        <v>0.8851429028936981</v>
+      </c>
+      <c r="J1861" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1861" t="inlineStr"/>
+    </row>
+    <row r="1862">
+      <c r="A1862" s="1" t="n">
+        <v>1860</v>
+      </c>
+      <c r="B1862" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0282.png</t>
+        </is>
+      </c>
+      <c r="C1862" t="inlineStr"/>
+      <c r="D1862" t="inlineStr"/>
+      <c r="E1862" t="inlineStr"/>
+      <c r="F1862" t="inlineStr">
+        <is>
+          <t>NC(=O)c1c(-c2ccc(Oc3ccccc3)cc2)nn2c1Nc1cc(C(=O)N3CCN(CC4CCN(c5ccc6c(c5)C(=O)N(C5CCC(=O)NC5=O)C6=O)CC4)CC3)ccc1CC2</t>
+        </is>
+      </c>
+      <c r="G1862" t="inlineStr"/>
+      <c r="H1862" t="inlineStr"/>
+      <c r="I1862" t="n">
+        <v>0.8768779745590215</v>
+      </c>
+      <c r="J1862" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1862" t="inlineStr"/>
+    </row>
+    <row r="1863">
+      <c r="A1863" s="1" t="n">
+        <v>1861</v>
+      </c>
+      <c r="B1863" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0283.png</t>
+        </is>
+      </c>
+      <c r="C1863" t="inlineStr"/>
+      <c r="D1863" t="inlineStr"/>
+      <c r="E1863" t="inlineStr"/>
+      <c r="F1863" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(CCCCCCN[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1863" t="inlineStr"/>
+      <c r="H1863" t="inlineStr"/>
+      <c r="I1863" t="n">
+        <v>0.8866901792044894</v>
+      </c>
+      <c r="J1863" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1863" t="inlineStr"/>
+    </row>
+    <row r="1864">
+      <c r="A1864" s="1" t="n">
+        <v>1862</v>
+      </c>
+      <c r="B1864" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0284.png</t>
+        </is>
+      </c>
+      <c r="C1864" t="inlineStr"/>
+      <c r="D1864" t="inlineStr"/>
+      <c r="E1864" t="inlineStr"/>
+      <c r="F1864" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCN(c2cc(C3=C4C=CC(=[N+](C)C)C=C4[Si](C)(C)c4cc(N(C)C)ccc43)c(C(=O)[O-])cc2OC)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1864" t="inlineStr"/>
+      <c r="H1864" t="inlineStr"/>
+      <c r="I1864" t="n">
+        <v>0.8959128187785722</v>
+      </c>
+      <c r="J1864" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1864" t="inlineStr"/>
+    </row>
+    <row r="1865">
+      <c r="A1865" s="1" t="n">
+        <v>1863</v>
+      </c>
+      <c r="B1865" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0285.png</t>
+        </is>
+      </c>
+      <c r="C1865" t="inlineStr"/>
+      <c r="D1865" t="inlineStr"/>
+      <c r="E1865" t="inlineStr"/>
+      <c r="F1865" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCC7CCN(C)C7)cc(O)c6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1865" t="inlineStr"/>
+      <c r="H1865" t="inlineStr"/>
+      <c r="I1865" t="n">
+        <v>0.8788828533668392</v>
+      </c>
+      <c r="J1865" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1865" t="inlineStr"/>
+    </row>
+    <row r="1866">
+      <c r="A1866" s="1" t="n">
+        <v>1864</v>
+      </c>
+      <c r="B1866" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0287.png</t>
+        </is>
+      </c>
+      <c r="C1866" t="inlineStr"/>
+      <c r="D1866" t="inlineStr"/>
+      <c r="E1866" t="inlineStr"/>
+      <c r="F1866" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccc2c(c1)CCCOc1cc(ccc1CC(=O)Nc1c(NC[C@H]3CCO3)cc(C(=O)OC)cc1OCCN(CC(F)(F)F)C(=O)OC(C)(C)C)-c1cccc(n1)OC2</t>
+        </is>
+      </c>
+      <c r="G1866" t="inlineStr"/>
+      <c r="H1866" t="inlineStr"/>
+      <c r="I1866" t="n">
+        <v>0.9034924523410569</v>
+      </c>
+      <c r="J1866" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1866" t="inlineStr"/>
+    </row>
+    <row r="1867">
+      <c r="A1867" s="1" t="n">
+        <v>1865</v>
+      </c>
+      <c r="B1867" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0289.png</t>
+        </is>
+      </c>
+      <c r="C1867" t="inlineStr"/>
+      <c r="D1867" t="inlineStr"/>
+      <c r="E1867" t="inlineStr"/>
+      <c r="F1867" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCCN)NC(=O)[C@H](CCCN)NCc2cccnc2Sc2c(F)ccc(-c3ccc(C(=O)O)cc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1867" t="inlineStr"/>
+      <c r="H1867" t="inlineStr"/>
+      <c r="I1867" t="n">
+        <v>0.8959456555453144</v>
+      </c>
+      <c r="J1867" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1867" t="inlineStr"/>
+    </row>
+    <row r="1868">
+      <c r="A1868" s="1" t="n">
+        <v>1866</v>
+      </c>
+      <c r="B1868" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0290.png</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr"/>
+      <c r="D1868" t="inlineStr"/>
+      <c r="E1868" t="inlineStr"/>
+      <c r="F1868" t="inlineStr">
+        <is>
+          <t>CC(C)c1cnn2c(NCc3ccccc3-c3nccc4cc(N5CCC(CN6CCN(c7ccc8c(c7)C(=O)N(C7CCC(=O)NC7=O)C8=O)CC6)CC5)ccc34)nc(O[C@@H]3CCCNC3)nc12</t>
+        </is>
+      </c>
+      <c r="G1868" t="inlineStr"/>
+      <c r="H1868" t="inlineStr"/>
+      <c r="I1868" t="n">
+        <v>0.8714307708154391</v>
+      </c>
+      <c r="J1868" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1868" t="inlineStr"/>
+    </row>
+    <row r="1869">
+      <c r="A1869" s="1" t="n">
+        <v>1867</v>
+      </c>
+      <c r="B1869" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0291.png</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr"/>
+      <c r="D1869" t="inlineStr"/>
+      <c r="E1869" t="inlineStr"/>
+      <c r="F1869" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc([C@H](C)NC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)c2cnc(C(=O)N3CCC(c4cc(Nc5cnccn5)nc(N5CCC(F)(F)C5)c4)CC3)cn2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1869" t="inlineStr"/>
+      <c r="H1869" t="inlineStr"/>
+      <c r="I1869" t="n">
+        <v>0.8966867677829597</v>
+      </c>
+      <c r="J1869" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1869" t="inlineStr"/>
+    </row>
+    <row r="1870">
+      <c r="A1870" s="1" t="n">
+        <v>1868</v>
+      </c>
+      <c r="B1870" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0292.png</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr"/>
+      <c r="D1870" t="inlineStr"/>
+      <c r="E1870" t="inlineStr"/>
+      <c r="F1870" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc([C@H](C)NC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)CN2CCN(c3cc(-c4ccccc4O)nnc3N)CC2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1870" t="inlineStr"/>
+      <c r="H1870" t="inlineStr"/>
+      <c r="I1870" t="n">
+        <v>0.8852395984020427</v>
+      </c>
+      <c r="J1870" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1870" t="inlineStr"/>
+    </row>
+    <row r="1871">
+      <c r="A1871" s="1" t="n">
+        <v>1869</v>
+      </c>
+      <c r="B1871" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0293.png</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr"/>
+      <c r="D1871" t="inlineStr"/>
+      <c r="E1871" t="inlineStr"/>
+      <c r="F1871" t="inlineStr">
+        <is>
+          <t>CC(C)c1cnn2c(NCc3ccccc3-c3nccc4cc(NC(=O)/C=C/CNCCOCCOCCNC(=O)CNc5cccc6c5C(=O)N(C5CCC(=O)NC5=O)C6=O)ccc34)nc(N3CCC(N)CC3)nc12</t>
+        </is>
+      </c>
+      <c r="G1871" t="inlineStr"/>
+      <c r="H1871" t="inlineStr"/>
+      <c r="I1871" t="n">
+        <v>0.894083720269331</v>
+      </c>
+      <c r="J1871" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1871" t="inlineStr"/>
+    </row>
+    <row r="1872">
+      <c r="A1872" s="1" t="n">
+        <v>1870</v>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0296.png</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr"/>
+      <c r="D1872" t="inlineStr"/>
+      <c r="E1872" t="inlineStr"/>
+      <c r="F1872" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccc2c(c1)CCCOc1cc(ccc1Cc1nc3c(OC4CCN(C)C4)cc(C(=O)OC)cc3n1C[C@@H]1CCO1)-c1cccc(n1)OC2</t>
+        </is>
+      </c>
+      <c r="G1872" t="inlineStr"/>
+      <c r="H1872" t="inlineStr"/>
+      <c r="I1872" t="n">
+        <v>0.9030797539313467</v>
+      </c>
+      <c r="J1872" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1872" t="inlineStr"/>
+    </row>
+    <row r="1873">
+      <c r="A1873" s="1" t="n">
+        <v>1871</v>
+      </c>
+      <c r="B1873" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0297.png</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr"/>
+      <c r="D1873" t="inlineStr"/>
+      <c r="E1873" t="inlineStr"/>
+      <c r="F1873" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCCN)NC(=O)[C@H](CCCN)NCc2nccnc2Sc2c(Cl)ccc(-c3ccc(C(=O)O)c(Cl)c3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1873" t="inlineStr"/>
+      <c r="H1873" t="inlineStr"/>
+      <c r="I1873" t="n">
+        <v>0.8959412946662736</v>
+      </c>
+      <c r="J1873" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1873" t="inlineStr"/>
+    </row>
+    <row r="1874">
+      <c r="A1874" s="1" t="n">
+        <v>1872</v>
+      </c>
+      <c r="B1874" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0298.png</t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr"/>
+      <c r="D1874" t="inlineStr"/>
+      <c r="E1874" t="inlineStr"/>
+      <c r="F1874" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2ccc(C3=C4C=CC(c5ccsc5)=[N+]4[B-](F)(F)n4c3ccc4-c3cccs3)cc2OC)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1874" t="inlineStr"/>
+      <c r="H1874" t="inlineStr"/>
+      <c r="I1874" t="n">
+        <v>0.8981512823968641</v>
+      </c>
+      <c r="J1874" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1874" t="inlineStr"/>
+    </row>
+    <row r="1875">
+      <c r="A1875" s="1" t="n">
+        <v>1873</v>
+      </c>
+      <c r="B1875" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0300.png</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr"/>
+      <c r="D1875" t="inlineStr"/>
+      <c r="E1875" t="inlineStr"/>
+      <c r="F1875" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN7CCOCC7)cc(O)c6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1875" t="inlineStr"/>
+      <c r="H1875" t="inlineStr"/>
+      <c r="I1875" t="n">
+        <v>0.8729541865878038</v>
+      </c>
+      <c r="J1875" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1875" t="inlineStr"/>
+    </row>
+    <row r="1876">
+      <c r="A1876" s="1" t="n">
+        <v>1874</v>
+      </c>
+      <c r="B1876" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0302.png</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr"/>
+      <c r="D1876" t="inlineStr"/>
+      <c r="E1876" t="inlineStr"/>
+      <c r="F1876" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCN)NC(=O)[C@H](CCCN)NCc2cccnc2Sc2c(F)ccc(-c3ccc(C(=O)O)nc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1876" t="inlineStr"/>
+      <c r="H1876" t="inlineStr"/>
+      <c r="I1876" t="n">
+        <v>0.8923639235173411</v>
+      </c>
+      <c r="J1876" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1876" t="inlineStr"/>
+    </row>
+    <row r="1877">
+      <c r="A1877" s="1" t="n">
+        <v>1875</v>
+      </c>
+      <c r="B1877" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0303.png</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr"/>
+      <c r="D1877" t="inlineStr"/>
+      <c r="E1877" t="inlineStr"/>
+      <c r="F1877" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)[C@@H]4C[C@@H]4C(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1877" t="inlineStr"/>
+      <c r="H1877" t="inlineStr"/>
+      <c r="I1877" t="n">
+        <v>0.8993212450228709</v>
+      </c>
+      <c r="J1877" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1877" t="inlineStr"/>
+    </row>
+    <row r="1878">
+      <c r="A1878" s="1" t="n">
+        <v>1876</v>
+      </c>
+      <c r="B1878" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0311.png</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr"/>
+      <c r="D1878" t="inlineStr"/>
+      <c r="E1878" t="inlineStr"/>
+      <c r="F1878" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCCN)NC(=O)[C@H](CCCN)NCc2cccnc2Sc2c(Cl)ccc(-c3ccc(C(=O)O)c(S(C)(=O)=O)c3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1878" t="inlineStr"/>
+      <c r="H1878" t="inlineStr"/>
+      <c r="I1878" t="n">
+        <v>0.8776819532721607</v>
+      </c>
+      <c r="J1878" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1878" t="inlineStr"/>
+    </row>
+    <row r="1879">
+      <c r="A1879" s="1" t="n">
+        <v>1877</v>
+      </c>
+      <c r="B1879" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0312.png</t>
+        </is>
+      </c>
+      <c r="C1879" t="inlineStr"/>
+      <c r="D1879" t="inlineStr"/>
+      <c r="E1879" t="inlineStr"/>
+      <c r="F1879" t="inlineStr">
+        <is>
+          <t>COc1cc2cc(c1OC)OCCCC(OC(=O)c1cc(Cl)c3cnn(Cc4ccccc4)c3c1)CCN1CCCN(CCCOC2=O)CC1</t>
+        </is>
+      </c>
+      <c r="G1879" t="inlineStr"/>
+      <c r="H1879" t="inlineStr"/>
+      <c r="I1879" t="n">
+        <v>0.9122290538689991</v>
+      </c>
+      <c r="J1879" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1879" t="inlineStr"/>
+    </row>
+    <row r="1880">
+      <c r="A1880" s="1" t="n">
+        <v>1878</v>
+      </c>
+      <c r="B1880" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0315.png</t>
+        </is>
+      </c>
+      <c r="C1880" t="inlineStr"/>
+      <c r="D1880" t="inlineStr"/>
+      <c r="E1880" t="inlineStr"/>
+      <c r="F1880" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN7CCOCC7)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1880" t="inlineStr"/>
+      <c r="H1880" t="inlineStr"/>
+      <c r="I1880" t="n">
+        <v>0.888994569840926</v>
+      </c>
+      <c r="J1880" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1880" t="inlineStr"/>
+    </row>
+    <row r="1881">
+      <c r="A1881" s="1" t="n">
+        <v>1879</v>
+      </c>
+      <c r="B1881" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0316.png</t>
+        </is>
+      </c>
+      <c r="C1881" t="inlineStr"/>
+      <c r="D1881" t="inlineStr"/>
+      <c r="E1881" t="inlineStr"/>
+      <c r="F1881" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1881" t="inlineStr"/>
+      <c r="H1881" t="inlineStr"/>
+      <c r="I1881" t="n">
+        <v>0.853807921961285</v>
+      </c>
+      <c r="J1881" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1881" t="inlineStr"/>
+    </row>
+    <row r="1882">
+      <c r="A1882" s="1" t="n">
+        <v>1880</v>
+      </c>
+      <c r="B1882" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0317.png</t>
+        </is>
+      </c>
+      <c r="C1882" t="inlineStr"/>
+      <c r="D1882" t="inlineStr"/>
+      <c r="E1882" t="inlineStr"/>
+      <c r="F1882" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)[C@@H]4CC[C@@H]4C(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1882" t="inlineStr"/>
+      <c r="H1882" t="inlineStr"/>
+      <c r="I1882" t="n">
+        <v>0.876555218355371</v>
+      </c>
+      <c r="J1882" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1882" t="inlineStr"/>
+    </row>
+    <row r="1883">
+      <c r="A1883" s="1" t="n">
+        <v>1881</v>
+      </c>
+      <c r="B1883" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0318.png</t>
+        </is>
+      </c>
+      <c r="C1883" t="inlineStr"/>
+      <c r="D1883" t="inlineStr"/>
+      <c r="E1883" t="inlineStr"/>
+      <c r="F1883" t="inlineStr">
+        <is>
+          <t>Cc1cc(-c2ncnc3[nH]c(-c4ccc(C5CCN(CC6CCN(c7ccc8c(c7)CN(C7CCC(=O)NC7=O)C8=O)CC6)CC5)cc4)cc23)ccc1CNC(=O)c1nc(C(C)(C)C)no1</t>
+        </is>
+      </c>
+      <c r="G1883" t="inlineStr"/>
+      <c r="H1883" t="inlineStr"/>
+      <c r="I1883" t="n">
+        <v>0.8790419124287648</v>
+      </c>
+      <c r="J1883" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1883" t="inlineStr"/>
+    </row>
+    <row r="1884">
+      <c r="A1884" s="1" t="n">
+        <v>1882</v>
+      </c>
+      <c r="B1884" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0321.png</t>
+        </is>
+      </c>
+      <c r="C1884" t="inlineStr"/>
+      <c r="D1884" t="inlineStr"/>
+      <c r="E1884" t="inlineStr"/>
+      <c r="F1884" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4cccc(CN[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)c4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1884" t="inlineStr"/>
+      <c r="H1884" t="inlineStr"/>
+      <c r="I1884" t="n">
+        <v>0.8633785271140404</v>
+      </c>
+      <c r="J1884" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1884" t="inlineStr"/>
+    </row>
+    <row r="1885">
+      <c r="A1885" s="1" t="n">
+        <v>1883</v>
+      </c>
+      <c r="B1885" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0322.png</t>
+        </is>
+      </c>
+      <c r="C1885" t="inlineStr"/>
+      <c r="D1885" t="inlineStr"/>
+      <c r="E1885" t="inlineStr"/>
+      <c r="F1885" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(Br)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1885" t="inlineStr"/>
+      <c r="H1885" t="inlineStr"/>
+      <c r="I1885" t="n">
+        <v>0.8913975425739714</v>
+      </c>
+      <c r="J1885" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1885" t="inlineStr"/>
+    </row>
+    <row r="1886">
+      <c r="A1886" s="1" t="n">
+        <v>1884</v>
+      </c>
+      <c r="B1886" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0323.png</t>
+        </is>
+      </c>
+      <c r="C1886" t="inlineStr"/>
+      <c r="D1886" t="inlineStr"/>
+      <c r="E1886" t="inlineStr"/>
+      <c r="F1886" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)c4cncc(C(=O)N[C@H](C(=O)N5C[C@H](O)C[C@H]5C(=O)N[C@@H](C)c5ccc(-c6scnc6C)cc5)C(C)(C)C)c4)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1886" t="inlineStr"/>
+      <c r="H1886" t="inlineStr"/>
+      <c r="I1886" t="n">
+        <v>0.8834369905332535</v>
+      </c>
+      <c r="J1886" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1886" t="inlineStr"/>
+    </row>
+    <row r="1887">
+      <c r="A1887" s="1" t="n">
+        <v>1885</v>
+      </c>
+      <c r="B1887" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0324.png</t>
+        </is>
+      </c>
+      <c r="C1887" t="inlineStr"/>
+      <c r="D1887" t="inlineStr"/>
+      <c r="E1887" t="inlineStr"/>
+      <c r="F1887" t="inlineStr">
+        <is>
+          <t>NC(=O)c1c(-c2ccc(Oc3ccccc3)cc2)nn2c1Nc1ccc(NC(=O)COCCOCCOCCOCCNc3cccc4c3C(=O)N(C3CCC(=O)NC3=O)C4=O)cc1CC2</t>
+        </is>
+      </c>
+      <c r="G1887" t="inlineStr"/>
+      <c r="H1887" t="inlineStr"/>
+      <c r="I1887" t="n">
+        <v>0.8721398559650142</v>
+      </c>
+      <c r="J1887" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1887" t="inlineStr"/>
+    </row>
+    <row r="1888">
+      <c r="A1888" s="1" t="n">
+        <v>1886</v>
+      </c>
+      <c r="B1888" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0326.png</t>
+        </is>
+      </c>
+      <c r="C1888" t="inlineStr"/>
+      <c r="D1888" t="inlineStr"/>
+      <c r="E1888" t="inlineStr"/>
+      <c r="F1888" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)[C@H]4C[C@H]4C(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1888" t="inlineStr"/>
+      <c r="H1888" t="inlineStr"/>
+      <c r="I1888" t="n">
+        <v>0.8996855566791238</v>
+      </c>
+      <c r="J1888" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1888" t="inlineStr"/>
+    </row>
+    <row r="1889">
+      <c r="A1889" s="1" t="n">
+        <v>1887</v>
+      </c>
+      <c r="B1889" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0328.png</t>
+        </is>
+      </c>
+      <c r="C1889" t="inlineStr"/>
+      <c r="D1889" t="inlineStr"/>
+      <c r="E1889" t="inlineStr"/>
+      <c r="F1889" t="inlineStr">
+        <is>
+          <t>Cc1cnc(Nc2cc(C3CCN(C4CC5(C4)CN(c4ccc6c(c4)C(=O)N(C4CCC(=O)NC4=O)C6=O)C5)CC3)cc(N3CCC(F)(F)C3)n2)cn1</t>
+        </is>
+      </c>
+      <c r="G1889" t="inlineStr"/>
+      <c r="H1889" t="inlineStr"/>
+      <c r="I1889" t="n">
+        <v>0.8873212995284203</v>
+      </c>
+      <c r="J1889" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1889" t="inlineStr"/>
+    </row>
+    <row r="1890">
+      <c r="A1890" s="1" t="n">
+        <v>1888</v>
+      </c>
+      <c r="B1890" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0330.png</t>
+        </is>
+      </c>
+      <c r="C1890" t="inlineStr"/>
+      <c r="D1890" t="inlineStr"/>
+      <c r="E1890" t="inlineStr"/>
+      <c r="F1890" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6ccc(Br)cc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1890" t="inlineStr"/>
+      <c r="H1890" t="inlineStr"/>
+      <c r="I1890" t="n">
+        <v>0.8769640720733435</v>
+      </c>
+      <c r="J1890" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1890" t="inlineStr"/>
+    </row>
+    <row r="1891">
+      <c r="A1891" s="1" t="n">
+        <v>1889</v>
+      </c>
+      <c r="B1891" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0333.png</t>
+        </is>
+      </c>
+      <c r="C1891" t="inlineStr"/>
+      <c r="D1891" t="inlineStr"/>
+      <c r="E1891" t="inlineStr"/>
+      <c r="F1891" t="inlineStr">
+        <is>
+          <t>CCOP(=O)(O)C(F)(F)c1ccc2[nH]c(C(=O)N[C@H]3CN(CCOCCOCCOCCNc4cccc5c4C(=O)N(C4CCC(=O)NC4=O)C5=O)CC[C@H]4CC[C@@H](C(=O)NCCNC(N)=O)N4C3=O)cc2c1</t>
+        </is>
+      </c>
+      <c r="G1891" t="inlineStr"/>
+      <c r="H1891" t="inlineStr"/>
+      <c r="I1891" t="n">
+        <v>0.8788099186918795</v>
+      </c>
+      <c r="J1891" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1891" t="inlineStr"/>
+    </row>
+    <row r="1892">
+      <c r="A1892" s="1" t="n">
+        <v>1890</v>
+      </c>
+      <c r="B1892" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0334.png</t>
+        </is>
+      </c>
+      <c r="C1892" t="inlineStr"/>
+      <c r="D1892" t="inlineStr"/>
+      <c r="E1892" t="inlineStr"/>
+      <c r="F1892" t="inlineStr">
+        <is>
+          <t>Cc1cc(-c2ncnc3[nH]c(-c4ccc(C5CCN(CC6CCN(c7cc8c(cc7F)C(=O)N(C7CCC(=O)NC7=O)C8=O)CC6)CC5)cc4)cc23)ccc1CNC(=O)c1nc(C(C)(C)C)no1</t>
+        </is>
+      </c>
+      <c r="G1892" t="inlineStr"/>
+      <c r="H1892" t="inlineStr"/>
+      <c r="I1892" t="n">
+        <v>0.8996394718333315</v>
+      </c>
+      <c r="J1892" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1892" t="inlineStr"/>
+    </row>
+    <row r="1893">
+      <c r="A1893" s="1" t="n">
+        <v>1891</v>
+      </c>
+      <c r="B1893" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0335.png</t>
+        </is>
+      </c>
+      <c r="C1893" t="inlineStr"/>
+      <c r="D1893" t="inlineStr"/>
+      <c r="E1893" t="inlineStr"/>
+      <c r="F1893" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN(C)C)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1893" t="inlineStr"/>
+      <c r="H1893" t="inlineStr"/>
+      <c r="I1893" t="n">
+        <v>0.8820637082942988</v>
+      </c>
+      <c r="J1893" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1893" t="inlineStr"/>
+    </row>
+    <row r="1894">
+      <c r="A1894" s="1" t="n">
+        <v>1892</v>
+      </c>
+      <c r="B1894" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0336.png</t>
+        </is>
+      </c>
+      <c r="C1894" t="inlineStr"/>
+      <c r="D1894" t="inlineStr"/>
+      <c r="E1894" t="inlineStr"/>
+      <c r="F1894" t="inlineStr">
+        <is>
+          <t>Cc1cnc(Nc2cc(C3CCN(CC4CCN(c5ccc6c(c5)C(=O)N(C5CCC(=O)NC5=O)C6=O)CC4)CC3)cc(N3CCC(F)(F)C3)n2)cn1</t>
+        </is>
+      </c>
+      <c r="G1894" t="inlineStr"/>
+      <c r="H1894" t="inlineStr"/>
+      <c r="I1894" t="n">
+        <v>0.9112476441011469</v>
+      </c>
+      <c r="J1894" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1894" t="inlineStr"/>
+    </row>
+    <row r="1895">
+      <c r="A1895" s="1" t="n">
+        <v>1893</v>
+      </c>
+      <c r="B1895" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0337.png</t>
+        </is>
+      </c>
+      <c r="C1895" t="inlineStr"/>
+      <c r="D1895" t="inlineStr"/>
+      <c r="E1895" t="inlineStr"/>
+      <c r="F1895" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccc2c(c1)CCCOc1cc(ccc1Cc1nc3c(OCC(=O)N(C)C)cc(C(=O)OC)cc3n1C[C@@H]1CCO1)-c1cccc(n1)OC2</t>
+        </is>
+      </c>
+      <c r="G1895" t="inlineStr"/>
+      <c r="H1895" t="inlineStr"/>
+      <c r="I1895" t="n">
+        <v>0.9058743949788565</v>
+      </c>
+      <c r="J1895" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1895" t="inlineStr"/>
+    </row>
+    <row r="1896">
+      <c r="A1896" s="1" t="n">
+        <v>1894</v>
+      </c>
+      <c r="B1896" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0338.png</t>
+        </is>
+      </c>
+      <c r="C1896" t="inlineStr"/>
+      <c r="D1896" t="inlineStr"/>
+      <c r="E1896" t="inlineStr"/>
+      <c r="F1896" t="inlineStr">
+        <is>
+          <t>CN1C(=O)[C@H](CCCN)NC(=O)[C@H](CCCN)NCc2cccnc2Sc2cccc(-c3ccc(C(=O)O)cc3)c2CNC(=O)[C@@H]1Cc1c[nH]c2ccccc12</t>
+        </is>
+      </c>
+      <c r="G1896" t="inlineStr"/>
+      <c r="H1896" t="inlineStr"/>
+      <c r="I1896" t="n">
+        <v>0.8862036901303013</v>
+      </c>
+      <c r="J1896" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1896" t="inlineStr"/>
+    </row>
+    <row r="1897">
+      <c r="A1897" s="1" t="n">
+        <v>1895</v>
+      </c>
+      <c r="B1897" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0339.png</t>
+        </is>
+      </c>
+      <c r="C1897" t="inlineStr"/>
+      <c r="D1897" t="inlineStr"/>
+      <c r="E1897" t="inlineStr"/>
+      <c r="F1897" t="inlineStr">
+        <is>
+          <t>COc1ccccc1N1CCOCCOCCN(c2cc3c(cc2OC)C2(OC3=O)c3cc(-c4ccncc4)c(OC(C)=O)cc3Oc3cc(OC(C)=O)c(-c4ccncc4)cc32)CCOCC1</t>
+        </is>
+      </c>
+      <c r="G1897" t="inlineStr"/>
+      <c r="H1897" t="inlineStr"/>
+      <c r="I1897" t="n">
+        <v>0.8872907072455989</v>
+      </c>
+      <c r="J1897" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1897" t="inlineStr"/>
+    </row>
+    <row r="1898">
+      <c r="A1898" s="1" t="n">
+        <v>1896</v>
+      </c>
+      <c r="B1898" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0341.png</t>
+        </is>
+      </c>
+      <c r="C1898" t="inlineStr"/>
+      <c r="D1898" t="inlineStr"/>
+      <c r="E1898" t="inlineStr"/>
+      <c r="F1898" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN(C)C)cc(OCc7ccccc7)c6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1898" t="inlineStr"/>
+      <c r="H1898" t="inlineStr"/>
+      <c r="I1898" t="n">
+        <v>0.8805210170181467</v>
+      </c>
+      <c r="J1898" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1898" t="inlineStr"/>
+    </row>
+    <row r="1899">
+      <c r="A1899" s="1" t="n">
+        <v>1897</v>
+      </c>
+      <c r="B1899" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0343.png</t>
+        </is>
+      </c>
+      <c r="C1899" t="inlineStr"/>
+      <c r="D1899" t="inlineStr"/>
+      <c r="E1899" t="inlineStr"/>
+      <c r="F1899" t="inlineStr">
+        <is>
+          <t>CCn1cncc1Cn1c(Cc2ccc3cc2OCCCc2cc(C#N)ccc2COc2cccc-3n2)nc2c(OC)cc(C(=O)OC)cc21</t>
+        </is>
+      </c>
+      <c r="G1899" t="inlineStr"/>
+      <c r="H1899" t="inlineStr"/>
+      <c r="I1899" t="n">
+        <v>0.907073236231128</v>
+      </c>
+      <c r="J1899" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1899" t="inlineStr"/>
+    </row>
+    <row r="1900">
+      <c r="A1900" s="1" t="n">
+        <v>1898</v>
+      </c>
+      <c r="B1900" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0344.png</t>
+        </is>
+      </c>
+      <c r="C1900" t="inlineStr"/>
+      <c r="D1900" t="inlineStr"/>
+      <c r="E1900" t="inlineStr"/>
+      <c r="F1900" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OC7CCNCC7)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1900" t="inlineStr"/>
+      <c r="H1900" t="inlineStr"/>
+      <c r="I1900" t="n">
+        <v>0.8897699710431715</v>
+      </c>
+      <c r="J1900" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1900" t="inlineStr"/>
+    </row>
+    <row r="1901">
+      <c r="A1901" s="1" t="n">
+        <v>1899</v>
+      </c>
+      <c r="B1901" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0345.png</t>
+        </is>
+      </c>
+      <c r="C1901" t="inlineStr"/>
+      <c r="D1901" t="inlineStr"/>
+      <c r="E1901" t="inlineStr"/>
+      <c r="F1901" t="inlineStr">
+        <is>
+          <t>Cc1ccc(-c2ccn(CC(=O)O)c(=O)c2)c2c1Sc1ncccc1CN[C@@H](CCCN)C(=O)N[C@@H](CCCCN)C(=O)N(C)[C@@H](Cc1c[nH]c3ccccc13)C(=O)NC2</t>
+        </is>
+      </c>
+      <c r="G1901" t="inlineStr"/>
+      <c r="H1901" t="inlineStr"/>
+      <c r="I1901" t="n">
+        <v>0.8799245958082826</v>
+      </c>
+      <c r="J1901" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1901" t="inlineStr"/>
+    </row>
+    <row r="1902">
+      <c r="A1902" s="1" t="n">
+        <v>1900</v>
+      </c>
+      <c r="B1902" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0346.png</t>
+        </is>
+      </c>
+      <c r="C1902" t="inlineStr"/>
+      <c r="D1902" t="inlineStr"/>
+      <c r="E1902" t="inlineStr"/>
+      <c r="F1902" t="inlineStr">
+        <is>
+          <t>[C-]#[N+]c1ccnc(Nc2cc(C3CCN(C(=O)[C@@H]4C[C@H]4C(=O)N[C@H](C(=O)N4C[C@H](O)C[C@H]4C(=O)N[C@@H](C)c4ccc(-c5scnc5C)cc4)C(C)(C)C)CC3)cc(N3CCC(F)(F)C3)n2)c1</t>
+        </is>
+      </c>
+      <c r="G1902" t="inlineStr"/>
+      <c r="H1902" t="inlineStr"/>
+      <c r="I1902" t="n">
+        <v>0.8823923113070917</v>
+      </c>
+      <c r="J1902" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1902" t="inlineStr"/>
+    </row>
+    <row r="1903">
+      <c r="A1903" s="1" t="n">
+        <v>1901</v>
+      </c>
+      <c r="B1903" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0347.png</t>
+        </is>
+      </c>
+      <c r="C1903" t="inlineStr"/>
+      <c r="D1903" t="inlineStr"/>
+      <c r="E1903" t="inlineStr"/>
+      <c r="F1903" t="inlineStr">
+        <is>
+          <t>CO[C@H]1/C=C/O[C@@]2(C)Oc3c(C)c(O)c4c(=O)c(c5oc6cc(OCCN(C)C(C)=O)ccc6nc-5c4c3C2=O)NC(=O)/C(C)=C\C=C\[C@H](C)[C@H](O)[C@@H](C)[C@@H](O)[C@@H](C)[C@H](OC(C)=O)[C@@H]1C</t>
+        </is>
+      </c>
+      <c r="G1903" t="inlineStr"/>
+      <c r="H1903" t="inlineStr"/>
+      <c r="I1903" t="n">
+        <v>0.8967818979303619</v>
+      </c>
+      <c r="J1903" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1903" t="inlineStr"/>
+    </row>
+    <row r="1904">
+      <c r="A1904" s="1" t="n">
+        <v>1902</v>
+      </c>
+      <c r="B1904" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0348.png</t>
+        </is>
+      </c>
+      <c r="C1904" t="inlineStr"/>
+      <c r="D1904" t="inlineStr"/>
+      <c r="E1904" t="inlineStr"/>
+      <c r="F1904" t="inlineStr">
+        <is>
+          <t>CC(C)c1cnn2c(NCc3ccccc3-c3nccc4cc(NCCOCCOCCNC(=O)CNc5cccc6c5C(=O)N(C5CCC(=O)NC5=O)C6=O)ccc34)nc(O[C@@H]3CCCNC3)nc12</t>
+        </is>
+      </c>
+      <c r="G1904" t="inlineStr"/>
+      <c r="H1904" t="inlineStr"/>
+      <c r="I1904" t="n">
+        <v>0.8531231849430729</v>
+      </c>
+      <c r="J1904" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1904" t="inlineStr"/>
+    </row>
+    <row r="1905">
+      <c r="A1905" s="1" t="n">
+        <v>1903</v>
+      </c>
+      <c r="B1905" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0349.png</t>
+        </is>
+      </c>
+      <c r="C1905" t="inlineStr"/>
+      <c r="D1905" t="inlineStr"/>
+      <c r="E1905" t="inlineStr"/>
+      <c r="F1905" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc(CNC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)c2ccnc(N3CCN(c4cc(-c5ccccc5O)nnc4N)CC3)c2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G1905" t="inlineStr"/>
+      <c r="H1905" t="inlineStr"/>
+      <c r="I1905" t="n">
+        <v>0.899499190477738</v>
+      </c>
+      <c r="J1905" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1905" t="inlineStr"/>
+    </row>
+    <row r="1906">
+      <c r="A1906" s="1" t="n">
+        <v>1904</v>
+      </c>
+      <c r="B1906" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T070712/rb_0350.png</t>
+        </is>
+      </c>
+      <c r="C1906" t="inlineStr"/>
+      <c r="D1906" t="inlineStr"/>
+      <c r="E1906" t="inlineStr"/>
+      <c r="F1906" t="inlineStr">
+        <is>
+          <t>O=C(O)c1ccc2nc(Cc3ccc4cc3OCCCc3cc(-n5ccc(=O)c(F)c5)ccc3COc3cccc-4n3)n(C[C@@H]3CCO3)c2c1</t>
+        </is>
+      </c>
+      <c r="G1906" t="inlineStr"/>
+      <c r="H1906" t="inlineStr"/>
+      <c r="I1906" t="n">
+        <v>0.9063762358982737</v>
+      </c>
+      <c r="J1906" t="inlineStr">
+        <is>
+          <t>High Confidence of SMILES being correct</t>
+        </is>
+      </c>
+      <c r="K1906" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>